<commit_message>
extracted weekly timetable offtimes
</commit_message>
<xml_diff>
--- a/data/BerkData2.xlsx
+++ b/data/BerkData2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e402f802124af4b/Masaüstü/Projects/Campus-Scheduling/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{C7D56005-EF58-47E5-AED3-01ACD5EC98BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D5575A5-7092-4576-B5D9-21BE74F4D00C}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D5C6F6-66CE-410A-B6E2-A36EE952E0AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-17640" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11020" yWindow="2630" windowWidth="22200" windowHeight="13700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="928" uniqueCount="437">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="435">
   <si>
     <t>DepartmentName</t>
   </si>
@@ -791,12 +791,6 @@
   </si>
   <si>
     <t>Kömür Jeolojisi</t>
-  </si>
-  <si>
-    <t>İNM 478</t>
-  </si>
-  <si>
-    <t>Köprü Mühendisliğine Giriş</t>
   </si>
   <si>
     <t>İNM 458</t>
@@ -1479,13 +1473,17 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}" name="Table1" displayName="Table1" ref="A1:H231" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
-  <autoFilter ref="A1:H231" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}" name="Table1" displayName="Table1" ref="A1:H230" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
+  <autoFilter ref="A1:H230" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="FİZ 168"/>
+        <filter val="FİZ 174"/>
+        <filter val="FİZ 176"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{E28ED7F9-92E9-43FB-898A-30B6DDD841D3}" name="DepartmentName" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{A24A0F99-F460-4F6A-BEC2-81C68341B7ED}" name="CourseCode" dataDxfId="6"/>
@@ -1785,18 +1783,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H231"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:H230"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.19921875" customWidth="1"/>
-    <col min="2" max="2" width="16.265625" customWidth="1"/>
-    <col min="3" max="3" width="24.796875" customWidth="1"/>
-    <col min="5" max="5" width="10.265625" customWidth="1"/>
-    <col min="6" max="6" width="16.59765625" customWidth="1"/>
-    <col min="7" max="7" width="14.19921875" customWidth="1"/>
+    <col min="1" max="1" width="22.1796875" customWidth="1"/>
+    <col min="2" max="2" width="16.26953125" customWidth="1"/>
+    <col min="3" max="3" width="24.81640625" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="16.6328125" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1819,10 +1817,10 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -1848,7 +1846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -1874,7 +1872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -1900,7 +1898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -1926,7 +1924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -1952,7 +1950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -1978,7 +1976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>24</v>
       </c>
@@ -2004,7 +2002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
@@ -2030,7 +2028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -2056,7 +2054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
@@ -2082,7 +2080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -2108,7 +2106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
@@ -2134,7 +2132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
@@ -2160,7 +2158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>21</v>
       </c>
@@ -2186,7 +2184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>21</v>
       </c>
@@ -2212,7 +2210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -2238,7 +2236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>27</v>
       </c>
@@ -2264,7 +2262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>24</v>
       </c>
@@ -2290,7 +2288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>21</v>
       </c>
@@ -2316,7 +2314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>24</v>
       </c>
@@ -2342,7 +2340,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>24</v>
       </c>
@@ -2368,7 +2366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
@@ -2394,7 +2392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>14</v>
       </c>
@@ -2420,7 +2418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -2446,7 +2444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>17</v>
       </c>
@@ -2472,7 +2470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>19</v>
       </c>
@@ -2498,7 +2496,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>21</v>
       </c>
@@ -2524,7 +2522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>17</v>
       </c>
@@ -2550,7 +2548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>27</v>
       </c>
@@ -2576,7 +2574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>19</v>
       </c>
@@ -2602,7 +2600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>27</v>
       </c>
@@ -2628,7 +2626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>21</v>
       </c>
@@ -2654,7 +2652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>19</v>
       </c>
@@ -2680,7 +2678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>21</v>
       </c>
@@ -2706,7 +2704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>17</v>
       </c>
@@ -2732,7 +2730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>7</v>
       </c>
@@ -2758,7 +2756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>7</v>
       </c>
@@ -2784,7 +2782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>27</v>
       </c>
@@ -2810,7 +2808,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>7</v>
       </c>
@@ -2836,7 +2834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>7</v>
       </c>
@@ -2862,7 +2860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>7</v>
       </c>
@@ -2888,7 +2886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>21</v>
       </c>
@@ -2914,7 +2912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>14</v>
       </c>
@@ -2940,7 +2938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>27</v>
       </c>
@@ -2966,7 +2964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>27</v>
       </c>
@@ -2992,7 +2990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>7</v>
       </c>
@@ -3018,7 +3016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>24</v>
       </c>
@@ -3044,7 +3042,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>27</v>
       </c>
@@ -3070,7 +3068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>7</v>
       </c>
@@ -3096,7 +3094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>21</v>
       </c>
@@ -3122,7 +3120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>21</v>
       </c>
@@ -3148,7 +3146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>24</v>
       </c>
@@ -3174,7 +3172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>7</v>
       </c>
@@ -3200,7 +3198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>24</v>
       </c>
@@ -3226,7 +3224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>14</v>
       </c>
@@ -3252,7 +3250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>19</v>
       </c>
@@ -3278,7 +3276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>21</v>
       </c>
@@ -3304,7 +3302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>21</v>
       </c>
@@ -3330,7 +3328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>21</v>
       </c>
@@ -3356,7 +3354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>21</v>
       </c>
@@ -3382,7 +3380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>21</v>
       </c>
@@ -3408,7 +3406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>24</v>
       </c>
@@ -3434,7 +3432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>21</v>
       </c>
@@ -3460,7 +3458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>27</v>
       </c>
@@ -3486,7 +3484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>14</v>
       </c>
@@ -3512,7 +3510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>19</v>
       </c>
@@ -3538,7 +3536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>24</v>
       </c>
@@ -3564,7 +3562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>21</v>
       </c>
@@ -3590,7 +3588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>21</v>
       </c>
@@ -3616,7 +3614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>7</v>
       </c>
@@ -3642,7 +3640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>24</v>
       </c>
@@ -3668,7 +3666,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>27</v>
       </c>
@@ -3694,7 +3692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>19</v>
       </c>
@@ -3720,7 +3718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>24</v>
       </c>
@@ -3746,7 +3744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>14</v>
       </c>
@@ -3772,7 +3770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>17</v>
       </c>
@@ -3798,7 +3796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>14</v>
       </c>
@@ -3824,7 +3822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>24</v>
       </c>
@@ -3850,7 +3848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>19</v>
       </c>
@@ -3876,7 +3874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>21</v>
       </c>
@@ -3902,7 +3900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>27</v>
       </c>
@@ -3928,7 +3926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>17</v>
       </c>
@@ -3954,7 +3952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>19</v>
       </c>
@@ -3980,7 +3978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>19</v>
       </c>
@@ -4006,7 +4004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>19</v>
       </c>
@@ -4032,7 +4030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>19</v>
       </c>
@@ -4058,7 +4056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>19</v>
       </c>
@@ -4084,7 +4082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>19</v>
       </c>
@@ -4110,7 +4108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>19</v>
       </c>
@@ -4136,7 +4134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>19</v>
       </c>
@@ -4162,7 +4160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>19</v>
       </c>
@@ -4188,7 +4186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>19</v>
       </c>
@@ -4214,7 +4212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>14</v>
       </c>
@@ -4240,7 +4238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>21</v>
       </c>
@@ -4266,7 +4264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>24</v>
       </c>
@@ -4292,7 +4290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>24</v>
       </c>
@@ -4318,7 +4316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>17</v>
       </c>
@@ -4344,7 +4342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>27</v>
       </c>
@@ -4370,7 +4368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>24</v>
       </c>
@@ -4396,7 +4394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>14</v>
       </c>
@@ -4422,7 +4420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>27</v>
       </c>
@@ -4448,7 +4446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>7</v>
       </c>
@@ -4474,7 +4472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>7</v>
       </c>
@@ -4500,7 +4498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>7</v>
       </c>
@@ -4526,7 +4524,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>7</v>
       </c>
@@ -4552,7 +4550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>7</v>
       </c>
@@ -4578,7 +4576,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>7</v>
       </c>
@@ -4604,7 +4602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>21</v>
       </c>
@@ -4630,7 +4628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>21</v>
       </c>
@@ -4656,7 +4654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>21</v>
       </c>
@@ -4682,7 +4680,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>24</v>
       </c>
@@ -4708,7 +4706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
         <v>24</v>
       </c>
@@ -4734,7 +4732,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>7</v>
       </c>
@@ -4760,7 +4758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
         <v>24</v>
       </c>
@@ -4786,7 +4784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
         <v>14</v>
       </c>
@@ -4812,7 +4810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>19</v>
       </c>
@@ -4838,7 +4836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>14</v>
       </c>
@@ -4864,7 +4862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>27</v>
       </c>
@@ -4890,7 +4888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>24</v>
       </c>
@@ -4916,7 +4914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="2" t="s">
         <v>24</v>
       </c>
@@ -4942,7 +4940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
         <v>17</v>
       </c>
@@ -4968,7 +4966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
         <v>17</v>
       </c>
@@ -4994,7 +4992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
         <v>17</v>
       </c>
@@ -5020,7 +5018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="2" t="s">
         <v>19</v>
       </c>
@@ -5046,7 +5044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>7</v>
       </c>
@@ -5072,7 +5070,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
         <v>14</v>
       </c>
@@ -5098,7 +5096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
         <v>27</v>
       </c>
@@ -5124,7 +5122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="2" t="s">
         <v>19</v>
       </c>
@@ -5150,7 +5148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
         <v>24</v>
       </c>
@@ -5176,7 +5174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
         <v>17</v>
       </c>
@@ -5202,7 +5200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
         <v>14</v>
       </c>
@@ -5219,18 +5217,18 @@
         <v>13</v>
       </c>
       <c r="F132" s="2">
-        <v>5213213</v>
+        <v>2587917</v>
       </c>
       <c r="G132" s="2">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="H132" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B133" s="2" t="s">
         <v>259</v>
@@ -5239,24 +5237,24 @@
         <v>260</v>
       </c>
       <c r="D133" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F133" s="2">
-        <v>2587917</v>
+        <v>4693090</v>
       </c>
       <c r="G133" s="2">
-        <v>20</v>
+        <v>135</v>
       </c>
       <c r="H133" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B134" s="2" t="s">
         <v>261</v>
@@ -5265,7 +5263,7 @@
         <v>262</v>
       </c>
       <c r="D134" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>10</v>
@@ -5274,15 +5272,15 @@
         <v>4693090</v>
       </c>
       <c r="G134" s="2">
-        <v>135</v>
+        <v>203</v>
       </c>
       <c r="H134" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B135" s="2" t="s">
         <v>263</v>
@@ -5297,24 +5295,24 @@
         <v>10</v>
       </c>
       <c r="F135" s="2">
-        <v>4693090</v>
+        <v>1041914</v>
       </c>
       <c r="G135" s="2">
-        <v>203</v>
+        <v>110</v>
       </c>
       <c r="H135" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B136" s="2" t="s">
         <v>265</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="D136" s="2">
         <v>1</v>
@@ -5326,39 +5324,39 @@
         <v>1041914</v>
       </c>
       <c r="G136" s="2">
-        <v>110</v>
+        <v>160</v>
       </c>
       <c r="H136" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B137" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="C137" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="C137" s="2" t="s">
-        <v>266</v>
-      </c>
       <c r="D137" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F137" s="2">
-        <v>1041914</v>
+        <v>3258742</v>
       </c>
       <c r="G137" s="2">
-        <v>160</v>
+        <v>9</v>
       </c>
       <c r="H137" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>17</v>
       </c>
@@ -5369,24 +5367,24 @@
         <v>269</v>
       </c>
       <c r="D138" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F138" s="2">
-        <v>3258742</v>
+        <v>3633158</v>
       </c>
       <c r="G138" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H138" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B139" s="2" t="s">
         <v>270</v>
@@ -5395,22 +5393,22 @@
         <v>271</v>
       </c>
       <c r="D139" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F139" s="2">
-        <v>3633158</v>
+        <v>1457877</v>
       </c>
       <c r="G139" s="2">
-        <v>8</v>
+        <v>74</v>
       </c>
       <c r="H139" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
         <v>24</v>
       </c>
@@ -5427,18 +5425,18 @@
         <v>10</v>
       </c>
       <c r="F140" s="2">
-        <v>1457877</v>
+        <v>2579557</v>
       </c>
       <c r="G140" s="2">
-        <v>74</v>
+        <v>117</v>
       </c>
       <c r="H140" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B141" s="2" t="s">
         <v>274</v>
@@ -5447,30 +5445,30 @@
         <v>275</v>
       </c>
       <c r="D141" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F141" s="2">
-        <v>2579557</v>
+        <v>2550816</v>
       </c>
       <c r="G141" s="2">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="H141" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B142" s="2" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C142" s="2" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="D142" s="2">
         <v>1</v>
@@ -5482,21 +5480,21 @@
         <v>2550816</v>
       </c>
       <c r="G142" s="2">
-        <v>102</v>
+        <v>15</v>
       </c>
       <c r="H142" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B143" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C143" s="2" t="s">
         <v>276</v>
-      </c>
-      <c r="C143" s="2" t="s">
-        <v>277</v>
       </c>
       <c r="D143" s="2">
         <v>1</v>
@@ -5505,24 +5503,24 @@
         <v>10</v>
       </c>
       <c r="F143" s="2">
-        <v>2550816</v>
+        <v>1739868</v>
       </c>
       <c r="G143" s="2">
-        <v>15</v>
+        <v>159</v>
       </c>
       <c r="H143" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B144" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="C144" s="2" t="s">
         <v>276</v>
-      </c>
-      <c r="C144" s="2" t="s">
-        <v>278</v>
       </c>
       <c r="D144" s="2">
         <v>1</v>
@@ -5531,21 +5529,21 @@
         <v>10</v>
       </c>
       <c r="F144" s="2">
-        <v>1739868</v>
+        <v>4117613</v>
       </c>
       <c r="G144" s="2">
-        <v>159</v>
+        <v>99</v>
       </c>
       <c r="H144" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B145" s="2" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C145" s="2" t="s">
         <v>278</v>
@@ -5557,24 +5555,24 @@
         <v>10</v>
       </c>
       <c r="F145" s="2">
-        <v>4117613</v>
+        <v>4828331</v>
       </c>
       <c r="G145" s="2">
-        <v>99</v>
+        <v>160</v>
       </c>
       <c r="H145" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D146" s="2">
         <v>1</v>
@@ -5583,24 +5581,24 @@
         <v>10</v>
       </c>
       <c r="F146" s="2">
-        <v>4828331</v>
+        <v>1875741</v>
       </c>
       <c r="G146" s="2">
-        <v>160</v>
+        <v>19</v>
       </c>
       <c r="H146" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="D147" s="2">
         <v>1</v>
@@ -5612,15 +5610,15 @@
         <v>1875741</v>
       </c>
       <c r="G147" s="2">
-        <v>19</v>
+        <v>189</v>
       </c>
       <c r="H147" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B148" s="2" t="s">
         <v>279</v>
@@ -5629,24 +5627,24 @@
         <v>280</v>
       </c>
       <c r="D148" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F148" s="2">
-        <v>1875741</v>
+        <v>1457877</v>
       </c>
       <c r="G148" s="2">
-        <v>189</v>
+        <v>19</v>
       </c>
       <c r="H148" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B149" s="2" t="s">
         <v>281</v>
@@ -5655,24 +5653,24 @@
         <v>282</v>
       </c>
       <c r="D149" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E149" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F149" s="2">
-        <v>1457877</v>
+        <v>1009202</v>
       </c>
       <c r="G149" s="2">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="H149" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B150" s="2" t="s">
         <v>283</v>
@@ -5681,24 +5679,24 @@
         <v>284</v>
       </c>
       <c r="D150" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E150" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F150" s="2">
-        <v>1009202</v>
+        <v>1267061</v>
       </c>
       <c r="G150" s="2">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="H150" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B151" s="2" t="s">
         <v>285</v>
@@ -5713,16 +5711,16 @@
         <v>13</v>
       </c>
       <c r="F151" s="2">
-        <v>1267061</v>
+        <v>3041802</v>
       </c>
       <c r="G151" s="2">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="H151" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="152" spans="1:8" x14ac:dyDescent="0.45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" s="2" t="s">
         <v>21</v>
       </c>
@@ -5733,24 +5731,24 @@
         <v>288</v>
       </c>
       <c r="D152" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E152" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F152" s="2">
-        <v>3041802</v>
+        <v>1121323</v>
       </c>
       <c r="G152" s="2">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H152" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B153" s="2" t="s">
         <v>289</v>
@@ -5759,24 +5757,24 @@
         <v>290</v>
       </c>
       <c r="D153" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E153" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F153" s="2">
-        <v>1121323</v>
+        <v>2028216</v>
       </c>
       <c r="G153" s="2">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="H153" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B154" s="2" t="s">
         <v>291</v>
@@ -5785,24 +5783,24 @@
         <v>292</v>
       </c>
       <c r="D154" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E154" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F154" s="2">
-        <v>2028216</v>
+        <v>1009202</v>
       </c>
       <c r="G154" s="2">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H154" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" s="2" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B155" s="2" t="s">
         <v>293</v>
@@ -5811,24 +5809,24 @@
         <v>294</v>
       </c>
       <c r="D155" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F155" s="2">
-        <v>1009202</v>
+        <v>3013005</v>
       </c>
       <c r="G155" s="2">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="H155" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>295</v>
@@ -5837,24 +5835,24 @@
         <v>296</v>
       </c>
       <c r="D156" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E156" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F156" s="2">
-        <v>3013005</v>
+        <v>2311022</v>
       </c>
       <c r="G156" s="2">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="H156" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B157" s="2" t="s">
         <v>297</v>
@@ -5863,24 +5861,24 @@
         <v>298</v>
       </c>
       <c r="D157" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E157" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F157" s="2">
-        <v>2311022</v>
+        <v>2391172</v>
       </c>
       <c r="G157" s="2">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="H157" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B158" s="2" t="s">
         <v>299</v>
@@ -5895,16 +5893,16 @@
         <v>10</v>
       </c>
       <c r="F158" s="2">
-        <v>2391172</v>
+        <v>1618088</v>
       </c>
       <c r="G158" s="2">
-        <v>80</v>
+        <v>99</v>
       </c>
       <c r="H158" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="2" t="s">
         <v>24</v>
       </c>
@@ -5921,7 +5919,7 @@
         <v>10</v>
       </c>
       <c r="F159" s="2">
-        <v>1618088</v>
+        <v>1235319</v>
       </c>
       <c r="G159" s="2">
         <v>99</v>
@@ -5930,7 +5928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" s="2" t="s">
         <v>24</v>
       </c>
@@ -5947,18 +5945,18 @@
         <v>10</v>
       </c>
       <c r="F160" s="2">
-        <v>1235319</v>
+        <v>2832797</v>
       </c>
       <c r="G160" s="2">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H160" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B161" s="2" t="s">
         <v>305</v>
@@ -5967,22 +5965,22 @@
         <v>306</v>
       </c>
       <c r="D161" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E161" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F161" s="2">
-        <v>2832797</v>
+        <v>3979315</v>
       </c>
       <c r="G161" s="2">
-        <v>97</v>
+        <v>20</v>
       </c>
       <c r="H161" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
         <v>14</v>
       </c>
@@ -5993,76 +5991,76 @@
         <v>308</v>
       </c>
       <c r="D162" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E162" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F162" s="2">
-        <v>3979315</v>
+        <v>3258742</v>
       </c>
       <c r="G162" s="2">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="H162" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="163" spans="1:8" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B163" s="2" t="s">
         <v>309</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="D163" s="2">
         <v>2</v>
       </c>
       <c r="E163" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F163" s="2">
-        <v>3258742</v>
+        <v>3070901</v>
       </c>
       <c r="G163" s="2">
-        <v>75</v>
+        <v>15</v>
       </c>
       <c r="H163" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B164" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="C164" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="C164" s="2" t="s">
-        <v>310</v>
-      </c>
       <c r="D164" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E164" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F164" s="2">
-        <v>3070901</v>
+        <v>3633158</v>
       </c>
       <c r="G164" s="2">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="H164" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B165" s="2" t="s">
         <v>312</v>
@@ -6071,24 +6069,24 @@
         <v>313</v>
       </c>
       <c r="D165" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E165" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F165" s="2">
-        <v>3633158</v>
+        <v>3850625</v>
       </c>
       <c r="G165" s="2">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="H165" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B166" s="2" t="s">
         <v>314</v>
@@ -6097,24 +6095,24 @@
         <v>315</v>
       </c>
       <c r="D166" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E166" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F166" s="2">
-        <v>3850625</v>
+        <v>4721220</v>
       </c>
       <c r="G166" s="2">
-        <v>97</v>
+        <v>144</v>
       </c>
       <c r="H166" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B167" s="2" t="s">
         <v>316</v>
@@ -6126,21 +6124,21 @@
         <v>3</v>
       </c>
       <c r="E167" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F167" s="2">
-        <v>4721220</v>
+        <v>1093367</v>
       </c>
       <c r="G167" s="2">
-        <v>144</v>
+        <v>39</v>
       </c>
       <c r="H167" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" s="2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B168" s="2" t="s">
         <v>318</v>
@@ -6149,24 +6147,24 @@
         <v>319</v>
       </c>
       <c r="D168" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E168" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F168" s="2">
-        <v>1093367</v>
+        <v>2238227</v>
       </c>
       <c r="G168" s="2">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="H168" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="B169" s="2" t="s">
         <v>320</v>
@@ -6181,18 +6179,18 @@
         <v>13</v>
       </c>
       <c r="F169" s="2">
-        <v>2238227</v>
+        <v>1086552</v>
       </c>
       <c r="G169" s="2">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="H169" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A170" s="2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B170" s="2" t="s">
         <v>322</v>
@@ -6201,82 +6199,82 @@
         <v>323</v>
       </c>
       <c r="D170" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E170" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F170" s="2">
-        <v>1086552</v>
+        <v>5320332</v>
       </c>
       <c r="G170" s="2">
-        <v>40</v>
+        <v>127</v>
       </c>
       <c r="H170" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B171" s="2" t="s">
         <v>324</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D171" s="2">
         <v>1</v>
       </c>
       <c r="E171" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F171" s="2">
-        <v>5320332</v>
+        <v>1830239</v>
       </c>
       <c r="G171" s="2">
-        <v>127</v>
+        <v>18</v>
       </c>
       <c r="H171" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B172" s="2" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="D172" s="2">
         <v>1</v>
       </c>
       <c r="E172" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F172" s="2">
-        <v>1830239</v>
+        <v>5320332</v>
       </c>
       <c r="G172" s="2">
-        <v>18</v>
+        <v>181</v>
       </c>
       <c r="H172" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D173" s="2">
         <v>1</v>
@@ -6288,21 +6286,21 @@
         <v>5320332</v>
       </c>
       <c r="G173" s="2">
-        <v>181</v>
+        <v>95</v>
       </c>
       <c r="H173" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B174" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="C174" s="2" t="s">
         <v>327</v>
-      </c>
-      <c r="C174" s="2" t="s">
-        <v>328</v>
       </c>
       <c r="D174" s="2">
         <v>1</v>
@@ -6314,39 +6312,39 @@
         <v>5320332</v>
       </c>
       <c r="G174" s="2">
-        <v>95</v>
+        <v>146</v>
       </c>
       <c r="H174" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C175" s="2" t="s">
         <v>329</v>
       </c>
       <c r="D175" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E175" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F175" s="2">
-        <v>5320332</v>
+        <v>1112262</v>
       </c>
       <c r="G175" s="2">
-        <v>146</v>
+        <v>55</v>
       </c>
       <c r="H175" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
         <v>21</v>
       </c>
@@ -6357,22 +6355,22 @@
         <v>331</v>
       </c>
       <c r="D176" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E176" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F176" s="2">
-        <v>1112262</v>
+        <v>1029126</v>
       </c>
       <c r="G176" s="2">
-        <v>55</v>
+        <v>128</v>
       </c>
       <c r="H176" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
         <v>21</v>
       </c>
@@ -6392,13 +6390,13 @@
         <v>1029126</v>
       </c>
       <c r="G177" s="2">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="H177" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
         <v>21</v>
       </c>
@@ -6409,24 +6407,24 @@
         <v>335</v>
       </c>
       <c r="D178" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E178" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F178" s="2">
-        <v>1029126</v>
+        <v>1932179</v>
       </c>
       <c r="G178" s="2">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="H178" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B179" s="2" t="s">
         <v>336</v>
@@ -6441,18 +6439,18 @@
         <v>13</v>
       </c>
       <c r="F179" s="2">
-        <v>1932179</v>
+        <v>2903204</v>
       </c>
       <c r="G179" s="2">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="H179" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="B180" s="2" t="s">
         <v>338</v>
@@ -6464,21 +6462,21 @@
         <v>4</v>
       </c>
       <c r="E180" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F180" s="2">
-        <v>2903204</v>
+        <v>1086552</v>
       </c>
       <c r="G180" s="2">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="H180" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B181" s="2" t="s">
         <v>340</v>
@@ -6490,21 +6488,21 @@
         <v>4</v>
       </c>
       <c r="E181" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F181" s="2">
-        <v>1086552</v>
+        <v>4321939</v>
       </c>
       <c r="G181" s="2">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="H181" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B182" s="2" t="s">
         <v>342</v>
@@ -6513,24 +6511,24 @@
         <v>343</v>
       </c>
       <c r="D182" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E182" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F182" s="2">
-        <v>4321939</v>
+        <v>2137934</v>
       </c>
       <c r="G182" s="2">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="H182" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B183" s="2" t="s">
         <v>344</v>
@@ -6539,24 +6537,24 @@
         <v>345</v>
       </c>
       <c r="D183" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E183" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F183" s="2">
-        <v>2137934</v>
+        <v>3371830</v>
       </c>
       <c r="G183" s="2">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="H183" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B184" s="2" t="s">
         <v>346</v>
@@ -6565,24 +6563,24 @@
         <v>347</v>
       </c>
       <c r="D184" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E184" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F184" s="2">
-        <v>3371830</v>
+        <v>2446060</v>
       </c>
       <c r="G184" s="2">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H184" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B185" s="2" t="s">
         <v>348</v>
@@ -6591,24 +6589,24 @@
         <v>349</v>
       </c>
       <c r="D185" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E185" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F185" s="2">
-        <v>2446060</v>
+        <v>2832797</v>
       </c>
       <c r="G185" s="2">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H185" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="186" spans="1:8" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B186" s="2" t="s">
         <v>350</v>
@@ -6617,7 +6615,7 @@
         <v>351</v>
       </c>
       <c r="D186" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E186" s="2" t="s">
         <v>13</v>
@@ -6626,21 +6624,21 @@
         <v>2832797</v>
       </c>
       <c r="G186" s="2">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H186" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="D187" s="2">
         <v>2</v>
@@ -6652,15 +6650,15 @@
         <v>2832797</v>
       </c>
       <c r="G187" s="2">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H187" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B188" s="2" t="s">
         <v>352</v>
@@ -6669,24 +6667,24 @@
         <v>353</v>
       </c>
       <c r="D188" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E188" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F188" s="2">
-        <v>2832797</v>
+        <v>4721220</v>
       </c>
       <c r="G188" s="2">
-        <v>6</v>
+        <v>73</v>
       </c>
       <c r="H188" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B189" s="2" t="s">
         <v>354</v>
@@ -6695,24 +6693,24 @@
         <v>355</v>
       </c>
       <c r="D189" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E189" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F189" s="2">
-        <v>4721220</v>
+        <v>7248701</v>
       </c>
       <c r="G189" s="2">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="H189" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="190" spans="1:8" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B190" s="2" t="s">
         <v>356</v>
@@ -6727,18 +6725,18 @@
         <v>13</v>
       </c>
       <c r="F190" s="2">
-        <v>7248701</v>
+        <v>2923606</v>
       </c>
       <c r="G190" s="2">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="H190" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B191" s="2" t="s">
         <v>358</v>
@@ -6747,24 +6745,24 @@
         <v>359</v>
       </c>
       <c r="D191" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E191" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F191" s="2">
-        <v>2923606</v>
+        <v>3143825</v>
       </c>
       <c r="G191" s="2">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="H191" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="192" spans="1:8" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="B192" s="2" t="s">
         <v>360</v>
@@ -6779,18 +6777,18 @@
         <v>10</v>
       </c>
       <c r="F192" s="2">
-        <v>3143825</v>
+        <v>5318224</v>
       </c>
       <c r="G192" s="2">
-        <v>84</v>
+        <v>54</v>
       </c>
       <c r="H192" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="193" spans="1:8" x14ac:dyDescent="0.45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" s="2" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="B193" s="2" t="s">
         <v>362</v>
@@ -6799,22 +6797,22 @@
         <v>363</v>
       </c>
       <c r="D193" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E193" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F193" s="2">
-        <v>5318224</v>
+        <v>3435711</v>
       </c>
       <c r="G193" s="2">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="H193" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" s="2" t="s">
         <v>7</v>
       </c>
@@ -6825,24 +6823,24 @@
         <v>365</v>
       </c>
       <c r="D194" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E194" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F194" s="2">
-        <v>3435711</v>
+        <v>1267061</v>
       </c>
       <c r="G194" s="2">
-        <v>42</v>
+        <v>102</v>
       </c>
       <c r="H194" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="195" spans="1:8" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="B195" s="2" t="s">
         <v>366</v>
@@ -6851,24 +6849,24 @@
         <v>367</v>
       </c>
       <c r="D195" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E195" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F195" s="2">
-        <v>1267061</v>
+        <v>2757489</v>
       </c>
       <c r="G195" s="2">
-        <v>102</v>
+        <v>43</v>
       </c>
       <c r="H195" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="196" spans="1:8" x14ac:dyDescent="0.45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="196" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>368</v>
@@ -6883,18 +6881,18 @@
         <v>13</v>
       </c>
       <c r="F196" s="2">
-        <v>2757489</v>
+        <v>2092090</v>
       </c>
       <c r="G196" s="2">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="H196" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B197" s="2" t="s">
         <v>370</v>
@@ -6903,24 +6901,24 @@
         <v>371</v>
       </c>
       <c r="D197" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E197" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F197" s="2">
-        <v>2092090</v>
+        <v>1707115</v>
       </c>
       <c r="G197" s="2">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="H197" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B198" s="2" t="s">
         <v>372</v>
@@ -6929,30 +6927,30 @@
         <v>373</v>
       </c>
       <c r="D198" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E198" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F198" s="2">
-        <v>1707115</v>
+        <v>1214802</v>
       </c>
       <c r="G198" s="2">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="H198" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A199" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>374</v>
       </c>
       <c r="C199" s="2" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="D199" s="2">
         <v>1</v>
@@ -6961,44 +6959,44 @@
         <v>10</v>
       </c>
       <c r="F199" s="2">
-        <v>1214802</v>
+        <v>2554019</v>
       </c>
       <c r="G199" s="2">
-        <v>97</v>
+        <v>141</v>
       </c>
       <c r="H199" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B200" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="C200" s="2" t="s">
         <v>376</v>
-      </c>
-      <c r="C200" s="2" t="s">
-        <v>375</v>
       </c>
       <c r="D200" s="2">
         <v>1</v>
       </c>
       <c r="E200" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F200" s="2">
-        <v>2554019</v>
+        <v>1098471</v>
       </c>
       <c r="G200" s="2">
-        <v>141</v>
+        <v>19</v>
       </c>
       <c r="H200" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B201" s="2" t="s">
         <v>377</v>
@@ -7007,24 +7005,24 @@
         <v>378</v>
       </c>
       <c r="D201" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E201" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F201" s="2">
-        <v>1098471</v>
+        <v>1410757</v>
       </c>
       <c r="G201" s="2">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="H201" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A202" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B202" s="2" t="s">
         <v>379</v>
@@ -7033,22 +7031,22 @@
         <v>380</v>
       </c>
       <c r="D202" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E202" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F202" s="2">
-        <v>1410757</v>
+        <v>1198965</v>
       </c>
       <c r="G202" s="2">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="H202" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
         <v>14</v>
       </c>
@@ -7065,18 +7063,18 @@
         <v>10</v>
       </c>
       <c r="F203" s="2">
-        <v>1198965</v>
+        <v>1561186</v>
       </c>
       <c r="G203" s="2">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H203" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A204" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B204" s="2" t="s">
         <v>383</v>
@@ -7088,21 +7086,21 @@
         <v>3</v>
       </c>
       <c r="E204" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F204" s="2">
-        <v>1561186</v>
+        <v>5475421</v>
       </c>
       <c r="G204" s="2">
-        <v>70</v>
+        <v>24</v>
       </c>
       <c r="H204" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A205" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B205" s="2" t="s">
         <v>385</v>
@@ -7111,24 +7109,24 @@
         <v>386</v>
       </c>
       <c r="D205" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E205" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F205" s="2">
-        <v>5475421</v>
+        <v>1235319</v>
       </c>
       <c r="G205" s="2">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="H205" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A206" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B206" s="2" t="s">
         <v>387</v>
@@ -7137,24 +7135,24 @@
         <v>388</v>
       </c>
       <c r="D206" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E206" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F206" s="2">
-        <v>1235319</v>
+        <v>1587825</v>
       </c>
       <c r="G206" s="2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H206" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B207" s="2" t="s">
         <v>389</v>
@@ -7163,24 +7161,24 @@
         <v>390</v>
       </c>
       <c r="D207" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E207" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F207" s="2">
-        <v>1587825</v>
+        <v>1235319</v>
       </c>
       <c r="G207" s="2">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H207" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="208" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A208" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B208" s="2" t="s">
         <v>391</v>
@@ -7189,24 +7187,24 @@
         <v>392</v>
       </c>
       <c r="D208" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E208" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F208" s="2">
-        <v>1235319</v>
+        <v>1047857</v>
       </c>
       <c r="G208" s="2">
-        <v>21</v>
+        <v>90</v>
       </c>
       <c r="H208" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="209" spans="1:8" x14ac:dyDescent="0.45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B209" s="2" t="s">
         <v>393</v>
@@ -7215,24 +7213,24 @@
         <v>394</v>
       </c>
       <c r="D209" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E209" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F209" s="2">
-        <v>1047857</v>
+        <v>1583231</v>
       </c>
       <c r="G209" s="2">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="H209" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="210" spans="1:8" x14ac:dyDescent="0.45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B210" s="2" t="s">
         <v>395</v>
@@ -7247,18 +7245,18 @@
         <v>10</v>
       </c>
       <c r="F210" s="2">
-        <v>1583231</v>
+        <v>2571190</v>
       </c>
       <c r="G210" s="2">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="H210" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A211" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B211" s="2" t="s">
         <v>397</v>
@@ -7267,56 +7265,56 @@
         <v>398</v>
       </c>
       <c r="D211" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E211" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F211" s="2">
-        <v>2571190</v>
+        <v>4205238</v>
       </c>
       <c r="G211" s="2">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="H211" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A212" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B212" s="2" t="s">
         <v>399</v>
       </c>
       <c r="C212" s="2" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
       <c r="D212" s="2">
         <v>2</v>
       </c>
       <c r="E212" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F212" s="2">
-        <v>4205238</v>
+        <v>5856415</v>
       </c>
       <c r="G212" s="2">
-        <v>18</v>
+        <v>91</v>
       </c>
       <c r="H212" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A213" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B213" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="C213" s="2" t="s">
         <v>401</v>
-      </c>
-      <c r="C213" s="2" t="s">
-        <v>400</v>
       </c>
       <c r="D213" s="2">
         <v>2</v>
@@ -7325,18 +7323,18 @@
         <v>10</v>
       </c>
       <c r="F213" s="2">
-        <v>5856415</v>
+        <v>2994200</v>
       </c>
       <c r="G213" s="2">
-        <v>91</v>
+        <v>131</v>
       </c>
       <c r="H213" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A214" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B214" s="2" t="s">
         <v>402</v>
@@ -7351,16 +7349,16 @@
         <v>10</v>
       </c>
       <c r="F214" s="2">
-        <v>2994200</v>
+        <v>2458943</v>
       </c>
       <c r="G214" s="2">
-        <v>131</v>
+        <v>105</v>
       </c>
       <c r="H214" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A215" s="2" t="s">
         <v>14</v>
       </c>
@@ -7371,24 +7369,24 @@
         <v>405</v>
       </c>
       <c r="D215" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E215" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F215" s="2">
-        <v>2458943</v>
+        <v>2234229</v>
       </c>
       <c r="G215" s="2">
-        <v>105</v>
+        <v>22</v>
       </c>
       <c r="H215" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A216" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B216" s="2" t="s">
         <v>406</v>
@@ -7403,18 +7401,18 @@
         <v>13</v>
       </c>
       <c r="F216" s="2">
-        <v>2234229</v>
+        <v>1410757</v>
       </c>
       <c r="G216" s="2">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="H216" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B217" s="2" t="s">
         <v>408</v>
@@ -7423,24 +7421,24 @@
         <v>409</v>
       </c>
       <c r="D217" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E217" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F217" s="2">
-        <v>1410757</v>
+        <v>5930518</v>
       </c>
       <c r="G217" s="2">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="H217" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B218" s="2" t="s">
         <v>410</v>
@@ -7449,24 +7447,24 @@
         <v>411</v>
       </c>
       <c r="D218" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E218" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F218" s="2">
-        <v>5930518</v>
+        <v>7208507</v>
       </c>
       <c r="G218" s="2">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="H218" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A219" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B219" s="2" t="s">
         <v>412</v>
@@ -7481,18 +7479,18 @@
         <v>13</v>
       </c>
       <c r="F219" s="2">
-        <v>7208507</v>
+        <v>1214802</v>
       </c>
       <c r="G219" s="2">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="H219" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A220" s="2" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B220" s="2" t="s">
         <v>414</v>
@@ -7501,24 +7499,24 @@
         <v>415</v>
       </c>
       <c r="D220" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E220" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F220" s="2">
-        <v>1214802</v>
+        <v>2002083</v>
       </c>
       <c r="G220" s="2">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="H220" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A221" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B221" s="2" t="s">
         <v>416</v>
@@ -7533,18 +7531,18 @@
         <v>13</v>
       </c>
       <c r="F221" s="2">
-        <v>2002083</v>
+        <v>5856415</v>
       </c>
       <c r="G221" s="2">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="H221" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="222" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A222" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B222" s="2" t="s">
         <v>418</v>
@@ -7553,24 +7551,24 @@
         <v>419</v>
       </c>
       <c r="D222" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E222" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F222" s="2">
-        <v>5856415</v>
+        <v>3334973</v>
       </c>
       <c r="G222" s="2">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="H222" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B223" s="2" t="s">
         <v>420</v>
@@ -7579,22 +7577,22 @@
         <v>421</v>
       </c>
       <c r="D223" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E223" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F223" s="2">
-        <v>3334973</v>
+        <v>5213213</v>
       </c>
       <c r="G223" s="2">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="H223" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A224" s="2" t="s">
         <v>14</v>
       </c>
@@ -7605,22 +7603,22 @@
         <v>423</v>
       </c>
       <c r="D224" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E224" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F224" s="2">
-        <v>5213213</v>
+        <v>1021641</v>
       </c>
       <c r="G224" s="2">
-        <v>24</v>
+        <v>130</v>
       </c>
       <c r="H224" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="225" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A225" s="2" t="s">
         <v>14</v>
       </c>
@@ -7637,18 +7635,18 @@
         <v>10</v>
       </c>
       <c r="F225" s="2">
-        <v>1021641</v>
+        <v>2092090</v>
       </c>
       <c r="G225" s="2">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H225" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A226" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B226" s="2" t="s">
         <v>426</v>
@@ -7657,24 +7655,24 @@
         <v>427</v>
       </c>
       <c r="D226" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E226" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F226" s="2">
-        <v>2092090</v>
+        <v>5997408</v>
       </c>
       <c r="G226" s="2">
-        <v>127</v>
+        <v>9</v>
       </c>
       <c r="H226" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="227" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A227" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B227" s="2" t="s">
         <v>428</v>
@@ -7686,19 +7684,19 @@
         <v>4</v>
       </c>
       <c r="E227" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F227" s="2">
-        <v>5997408</v>
+        <v>3524624</v>
       </c>
       <c r="G227" s="2">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="H227" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="228" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A228" s="2" t="s">
         <v>14</v>
       </c>
@@ -7709,30 +7707,30 @@
         <v>431</v>
       </c>
       <c r="D228" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E228" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F228" s="2">
-        <v>3524624</v>
+        <v>1892200</v>
       </c>
       <c r="G228" s="2">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="H228" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="229" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A229" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B229" s="2" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C229" s="2" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="D229" s="2">
         <v>3</v>
@@ -7744,15 +7742,15 @@
         <v>1892200</v>
       </c>
       <c r="G229" s="2">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H229" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="230" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A230" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B230" s="2" t="s">
         <v>432</v>
@@ -7764,41 +7762,15 @@
         <v>3</v>
       </c>
       <c r="E230" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F230" s="2">
-        <v>1892200</v>
+        <v>2977082</v>
       </c>
       <c r="G230" s="2">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="H230" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="231" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A231" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B231" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="C231" s="2" t="s">
-        <v>435</v>
-      </c>
-      <c r="D231" s="2">
-        <v>3</v>
-      </c>
-      <c r="E231" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F231" s="2">
-        <v>2977082</v>
-      </c>
-      <c r="G231" s="2">
-        <v>52</v>
-      </c>
-      <c r="H231" s="2">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
timetable offtimes implemented. TODO: investigate statistics
</commit_message>
<xml_diff>
--- a/data/BerkData2.xlsx
+++ b/data/BerkData2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90D5C6F6-66CE-410A-B6E2-A36EE952E0AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E762A5A-9DFC-4DD5-AE62-7B921CAD2900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11020" yWindow="2630" windowWidth="22200" windowHeight="13700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-37965" yWindow="9300" windowWidth="22200" windowHeight="10875" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1475,15 +1475,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}" name="Table1" displayName="Table1" ref="A1:H230" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
-  <autoFilter ref="A1:H230" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="FİZ 168"/>
-        <filter val="FİZ 174"/>
-        <filter val="FİZ 176"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:H230" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{E28ED7F9-92E9-43FB-898A-30B6DDD841D3}" name="DepartmentName" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{A24A0F99-F460-4F6A-BEC2-81C68341B7ED}" name="CourseCode" dataDxfId="6"/>
@@ -1820,7 +1812,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -1846,7 +1838,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -1872,7 +1864,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -1898,7 +1890,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -1924,7 +1916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -1950,7 +1942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -1976,7 +1968,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>24</v>
       </c>
@@ -2002,7 +1994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
@@ -2028,7 +2020,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -2054,7 +2046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
@@ -2080,7 +2072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -2106,7 +2098,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
@@ -2132,7 +2124,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
@@ -2158,7 +2150,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>21</v>
       </c>
@@ -2184,7 +2176,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>21</v>
       </c>
@@ -2210,7 +2202,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -2236,7 +2228,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>27</v>
       </c>
@@ -2262,7 +2254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>24</v>
       </c>
@@ -2288,7 +2280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>21</v>
       </c>
@@ -2314,7 +2306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>24</v>
       </c>
@@ -2340,7 +2332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>24</v>
       </c>
@@ -2366,7 +2358,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
@@ -2392,7 +2384,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>14</v>
       </c>
@@ -2418,7 +2410,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -2444,7 +2436,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>17</v>
       </c>
@@ -2470,7 +2462,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>19</v>
       </c>
@@ -2496,7 +2488,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>21</v>
       </c>
@@ -2522,7 +2514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>17</v>
       </c>
@@ -2548,7 +2540,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>27</v>
       </c>
@@ -2574,7 +2566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>19</v>
       </c>
@@ -2600,7 +2592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>27</v>
       </c>
@@ -2626,7 +2618,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>21</v>
       </c>
@@ -2652,7 +2644,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>19</v>
       </c>
@@ -2678,7 +2670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>21</v>
       </c>
@@ -2704,7 +2696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>17</v>
       </c>
@@ -2730,7 +2722,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>7</v>
       </c>
@@ -2756,7 +2748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>7</v>
       </c>
@@ -2782,7 +2774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>27</v>
       </c>
@@ -2808,7 +2800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>7</v>
       </c>
@@ -2834,7 +2826,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>7</v>
       </c>
@@ -2860,7 +2852,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>7</v>
       </c>
@@ -2886,7 +2878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>21</v>
       </c>
@@ -2912,7 +2904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>14</v>
       </c>
@@ -2938,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>27</v>
       </c>
@@ -2964,7 +2956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>27</v>
       </c>
@@ -2990,7 +2982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>7</v>
       </c>
@@ -3016,7 +3008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>24</v>
       </c>
@@ -3042,7 +3034,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>27</v>
       </c>
@@ -3068,7 +3060,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>7</v>
       </c>
@@ -3094,7 +3086,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>21</v>
       </c>
@@ -3120,7 +3112,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>21</v>
       </c>
@@ -3146,7 +3138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>24</v>
       </c>
@@ -3172,7 +3164,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>7</v>
       </c>
@@ -3198,7 +3190,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>24</v>
       </c>
@@ -3224,7 +3216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>14</v>
       </c>
@@ -3250,7 +3242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>19</v>
       </c>
@@ -3276,7 +3268,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>21</v>
       </c>
@@ -3302,7 +3294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>21</v>
       </c>
@@ -3328,7 +3320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>21</v>
       </c>
@@ -3354,7 +3346,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>21</v>
       </c>
@@ -3380,7 +3372,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>21</v>
       </c>
@@ -3406,7 +3398,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>24</v>
       </c>
@@ -3432,7 +3424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>21</v>
       </c>
@@ -3458,7 +3450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>27</v>
       </c>
@@ -3484,7 +3476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>14</v>
       </c>
@@ -3510,7 +3502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>19</v>
       </c>
@@ -3536,7 +3528,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>24</v>
       </c>
@@ -3562,7 +3554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>21</v>
       </c>
@@ -3588,7 +3580,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>21</v>
       </c>
@@ -3614,7 +3606,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>7</v>
       </c>
@@ -3640,7 +3632,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>24</v>
       </c>
@@ -3666,7 +3658,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>27</v>
       </c>
@@ -3692,7 +3684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>19</v>
       </c>
@@ -3718,7 +3710,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>24</v>
       </c>
@@ -3744,7 +3736,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>14</v>
       </c>
@@ -3770,7 +3762,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>17</v>
       </c>
@@ -3822,7 +3814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>24</v>
       </c>
@@ -3874,7 +3866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>21</v>
       </c>
@@ -3900,7 +3892,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>27</v>
       </c>
@@ -3926,7 +3918,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>17</v>
       </c>
@@ -3952,7 +3944,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>19</v>
       </c>
@@ -3978,7 +3970,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>19</v>
       </c>
@@ -4004,7 +3996,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>19</v>
       </c>
@@ -4030,7 +4022,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>19</v>
       </c>
@@ -4056,7 +4048,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>19</v>
       </c>
@@ -4082,7 +4074,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>19</v>
       </c>
@@ -4108,7 +4100,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>19</v>
       </c>
@@ -4134,7 +4126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>19</v>
       </c>
@@ -4160,7 +4152,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>19</v>
       </c>
@@ -4186,7 +4178,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>19</v>
       </c>
@@ -4212,7 +4204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>14</v>
       </c>
@@ -4238,7 +4230,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>21</v>
       </c>
@@ -4264,7 +4256,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>24</v>
       </c>
@@ -4290,7 +4282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>24</v>
       </c>
@@ -4316,7 +4308,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>17</v>
       </c>
@@ -4342,7 +4334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>27</v>
       </c>
@@ -4368,7 +4360,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>24</v>
       </c>
@@ -4394,7 +4386,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>14</v>
       </c>
@@ -4420,7 +4412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>27</v>
       </c>
@@ -4446,7 +4438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>7</v>
       </c>
@@ -4472,7 +4464,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>7</v>
       </c>
@@ -4498,7 +4490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>7</v>
       </c>
@@ -4524,7 +4516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>7</v>
       </c>
@@ -4550,7 +4542,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>7</v>
       </c>
@@ -4576,7 +4568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>7</v>
       </c>
@@ -4602,7 +4594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>21</v>
       </c>
@@ -4628,7 +4620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>21</v>
       </c>
@@ -4654,7 +4646,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>21</v>
       </c>
@@ -4680,7 +4672,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>24</v>
       </c>
@@ -4706,7 +4698,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
         <v>24</v>
       </c>
@@ -4732,7 +4724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>7</v>
       </c>
@@ -4758,7 +4750,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
         <v>24</v>
       </c>
@@ -4784,7 +4776,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
         <v>14</v>
       </c>
@@ -4810,7 +4802,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>19</v>
       </c>
@@ -4836,7 +4828,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>14</v>
       </c>
@@ -4862,7 +4854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>27</v>
       </c>
@@ -4888,7 +4880,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>24</v>
       </c>
@@ -4914,7 +4906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A121" s="2" t="s">
         <v>24</v>
       </c>
@@ -4940,7 +4932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
         <v>17</v>
       </c>
@@ -4966,7 +4958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
         <v>17</v>
       </c>
@@ -4992,7 +4984,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
         <v>17</v>
       </c>
@@ -5018,7 +5010,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A125" s="2" t="s">
         <v>19</v>
       </c>
@@ -5044,7 +5036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>7</v>
       </c>
@@ -5070,7 +5062,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
         <v>14</v>
       </c>
@@ -5096,7 +5088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
         <v>27</v>
       </c>
@@ -5122,7 +5114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A129" s="2" t="s">
         <v>19</v>
       </c>
@@ -5148,7 +5140,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
         <v>24</v>
       </c>
@@ -5174,7 +5166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
         <v>17</v>
       </c>
@@ -5200,7 +5192,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
         <v>14</v>
       </c>
@@ -5226,7 +5218,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
         <v>7</v>
       </c>
@@ -5252,7 +5244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
         <v>21</v>
       </c>
@@ -5278,7 +5270,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" s="2" t="s">
         <v>14</v>
       </c>
@@ -5304,7 +5296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
         <v>24</v>
       </c>
@@ -5330,7 +5322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
         <v>17</v>
       </c>
@@ -5356,7 +5348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>17</v>
       </c>
@@ -5382,7 +5374,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" s="2" t="s">
         <v>24</v>
       </c>
@@ -5408,7 +5400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
         <v>24</v>
       </c>
@@ -5434,7 +5426,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A141" s="2" t="s">
         <v>14</v>
       </c>
@@ -5460,7 +5452,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A142" s="2" t="s">
         <v>17</v>
       </c>
@@ -5486,7 +5478,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A143" s="2" t="s">
         <v>24</v>
       </c>
@@ -5512,7 +5504,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
         <v>19</v>
       </c>
@@ -5538,7 +5530,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A145" s="2" t="s">
         <v>7</v>
       </c>
@@ -5564,7 +5556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
         <v>27</v>
       </c>
@@ -5590,7 +5582,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A147" s="2" t="s">
         <v>21</v>
       </c>
@@ -5616,7 +5608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A148" s="2" t="s">
         <v>24</v>
       </c>
@@ -5642,7 +5634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A149" s="2" t="s">
         <v>17</v>
       </c>
@@ -5668,7 +5660,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
         <v>7</v>
       </c>
@@ -5694,7 +5686,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
         <v>21</v>
       </c>
@@ -5720,7 +5712,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A152" s="2" t="s">
         <v>21</v>
       </c>
@@ -5746,7 +5738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
         <v>14</v>
       </c>
@@ -5772,7 +5764,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A154" s="2" t="s">
         <v>17</v>
       </c>
@@ -5798,7 +5790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A155" s="2" t="s">
         <v>7</v>
       </c>
@@ -5824,7 +5816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
         <v>19</v>
       </c>
@@ -5850,7 +5842,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
         <v>14</v>
       </c>
@@ -5876,7 +5868,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
         <v>24</v>
       </c>
@@ -5902,7 +5894,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A159" s="2" t="s">
         <v>24</v>
       </c>
@@ -5928,7 +5920,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A160" s="2" t="s">
         <v>24</v>
       </c>
@@ -5954,7 +5946,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
         <v>14</v>
       </c>
@@ -5980,7 +5972,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
         <v>14</v>
       </c>
@@ -6006,7 +5998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
         <v>27</v>
       </c>
@@ -6032,7 +6024,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
         <v>17</v>
       </c>
@@ -6058,7 +6050,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
         <v>19</v>
       </c>
@@ -6084,7 +6076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A166" s="2" t="s">
         <v>21</v>
       </c>
@@ -6110,7 +6102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A167" s="2" t="s">
         <v>19</v>
       </c>
@@ -6136,7 +6128,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A168" s="2" t="s">
         <v>7</v>
       </c>
@@ -6162,7 +6154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A169" s="2" t="s">
         <v>19</v>
       </c>
@@ -6214,7 +6206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
         <v>27</v>
       </c>
@@ -6318,7 +6310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A175" s="2" t="s">
         <v>21</v>
       </c>
@@ -6344,7 +6336,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
         <v>21</v>
       </c>
@@ -6370,7 +6362,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
         <v>21</v>
       </c>
@@ -6396,7 +6388,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
         <v>21</v>
       </c>
@@ -6422,7 +6414,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A179" s="2" t="s">
         <v>7</v>
       </c>
@@ -6448,7 +6440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
         <v>19</v>
       </c>
@@ -6474,7 +6466,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
         <v>21</v>
       </c>
@@ -6500,7 +6492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
         <v>19</v>
       </c>
@@ -6526,7 +6518,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
         <v>24</v>
       </c>
@@ -6552,7 +6544,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A184" s="2" t="s">
         <v>17</v>
       </c>
@@ -6578,7 +6570,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A185" s="2" t="s">
         <v>24</v>
       </c>
@@ -6604,7 +6596,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A186" s="2" t="s">
         <v>27</v>
       </c>
@@ -6630,7 +6622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
         <v>17</v>
       </c>
@@ -6656,7 +6648,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
         <v>21</v>
       </c>
@@ -6682,7 +6674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
         <v>7</v>
       </c>
@@ -6708,7 +6700,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
         <v>21</v>
       </c>
@@ -6734,7 +6726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
         <v>7</v>
       </c>
@@ -6760,7 +6752,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
         <v>24</v>
       </c>
@@ -6786,7 +6778,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A193" s="2" t="s">
         <v>7</v>
       </c>
@@ -6812,7 +6804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A194" s="2" t="s">
         <v>7</v>
       </c>
@@ -6838,7 +6830,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A195" s="2" t="s">
         <v>19</v>
       </c>
@@ -6864,7 +6856,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
         <v>14</v>
       </c>
@@ -6890,7 +6882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
         <v>24</v>
       </c>
@@ -6916,7 +6908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
         <v>14</v>
       </c>
@@ -6942,7 +6934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A199" s="2" t="s">
         <v>24</v>
       </c>
@@ -6968,7 +6960,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
         <v>27</v>
       </c>
@@ -6994,7 +6986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
         <v>17</v>
       </c>
@@ -7020,7 +7012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A202" s="2" t="s">
         <v>14</v>
       </c>
@@ -7046,7 +7038,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
         <v>14</v>
       </c>
@@ -7072,7 +7064,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A204" s="2" t="s">
         <v>19</v>
       </c>
@@ -7098,7 +7090,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A205" s="2" t="s">
         <v>24</v>
       </c>
@@ -7124,7 +7116,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A206" s="2" t="s">
         <v>27</v>
       </c>
@@ -7150,7 +7142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
         <v>24</v>
       </c>
@@ -7176,7 +7168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A208" s="2" t="s">
         <v>19</v>
       </c>
@@ -7202,7 +7194,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
         <v>14</v>
       </c>
@@ -7228,7 +7220,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
         <v>19</v>
       </c>
@@ -7254,7 +7246,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A211" s="2" t="s">
         <v>27</v>
       </c>
@@ -7280,7 +7272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A212" s="2" t="s">
         <v>19</v>
       </c>
@@ -7306,7 +7298,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A213" s="2" t="s">
         <v>24</v>
       </c>
@@ -7332,7 +7324,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A214" s="2" t="s">
         <v>14</v>
       </c>
@@ -7358,7 +7350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A215" s="2" t="s">
         <v>14</v>
       </c>
@@ -7384,7 +7376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A216" s="2" t="s">
         <v>17</v>
       </c>
@@ -7410,7 +7402,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A217" s="2" t="s">
         <v>19</v>
       </c>
@@ -7436,7 +7428,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
         <v>21</v>
       </c>
@@ -7462,7 +7454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A219" s="2" t="s">
         <v>14</v>
       </c>
@@ -7488,7 +7480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A220" s="2" t="s">
         <v>27</v>
       </c>
@@ -7514,7 +7506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A221" s="2" t="s">
         <v>19</v>
       </c>
@@ -7540,7 +7532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A222" s="2" t="s">
         <v>24</v>
       </c>
@@ -7566,7 +7558,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
         <v>14</v>
       </c>
@@ -7592,7 +7584,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A224" s="2" t="s">
         <v>14</v>
       </c>
@@ -7618,7 +7610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A225" s="2" t="s">
         <v>14</v>
       </c>
@@ -7644,7 +7636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A226" s="2" t="s">
         <v>17</v>
       </c>
@@ -7670,7 +7662,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A227" s="2" t="s">
         <v>14</v>
       </c>
@@ -7696,7 +7688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A228" s="2" t="s">
         <v>14</v>
       </c>
@@ -7722,7 +7714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="229" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A229" s="2" t="s">
         <v>17</v>
       </c>
@@ -7748,7 +7740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="230" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A230" s="2" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
analysis preprocessing done. TODO: find performance metrics
</commit_message>
<xml_diff>
--- a/data/BerkData2.xlsx
+++ b/data/BerkData2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8E97416-06D2-4CF7-8C37-54F8A6A9B715}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{771F3311-E453-48DD-94B7-640279B5D8D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1476,9 +1476,9 @@
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}" name="Table1" displayName="Table1" ref="A1:H228" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
   <autoFilter ref="A1:H228" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}">
-    <filterColumn colId="0">
+    <filterColumn colId="1">
       <filters>
-        <filter val="Elektrik-Elektronik Mühendisliği"/>
+        <filter val="İNM 108"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -1948,7 +1948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -2130,7 +2130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
@@ -2156,7 +2156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>21</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>21</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>21</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>21</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>21</v>
       </c>
@@ -2676,7 +2676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>21</v>
       </c>
@@ -2884,7 +2884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>21</v>
       </c>
@@ -3092,7 +3092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>21</v>
       </c>
@@ -3118,7 +3118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>21</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>21</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>21</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>21</v>
       </c>
@@ -3352,7 +3352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>21</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>21</v>
       </c>
@@ -3430,7 +3430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>21</v>
       </c>
@@ -3560,7 +3560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>21</v>
       </c>
@@ -3586,7 +3586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>21</v>
       </c>
@@ -3742,7 +3742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>14</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>17</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>21</v>
       </c>
@@ -4210,7 +4210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>21</v>
       </c>
@@ -4574,7 +4574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>21</v>
       </c>
@@ -4600,7 +4600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>21</v>
       </c>
@@ -4626,7 +4626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>21</v>
       </c>
@@ -5224,7 +5224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
         <v>21</v>
       </c>
@@ -5562,7 +5562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
         <v>21</v>
       </c>
@@ -5666,7 +5666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
         <v>21</v>
       </c>
@@ -5692,7 +5692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
         <v>21</v>
       </c>
@@ -6056,7 +6056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
         <v>21</v>
       </c>
@@ -6212,7 +6212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
         <v>21</v>
       </c>
@@ -6264,7 +6264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
         <v>21</v>
       </c>
@@ -6290,7 +6290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
         <v>21</v>
       </c>
@@ -6316,7 +6316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" s="2" t="s">
         <v>21</v>
       </c>
@@ -6342,7 +6342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
         <v>21</v>
       </c>
@@ -6368,7 +6368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
         <v>21</v>
       </c>
@@ -6446,7 +6446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
         <v>21</v>
       </c>
@@ -6628,7 +6628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
         <v>21</v>
       </c>
@@ -6680,7 +6680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
         <v>21</v>
       </c>
@@ -7408,7 +7408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
       <c r="A217" s="2" t="s">
         <v>21</v>
       </c>

</xml_diff>

<commit_message>
department manuel schedules done
</commit_message>
<xml_diff>
--- a/data/BerkData2.xlsx
+++ b/data/BerkData2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e402f802124af4b/Masaüstü/Projects/Campus-Scheduling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C943E96-C6E4-40C4-888D-FAADD3A22539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{2C943E96-C6E4-40C4-888D-FAADD3A22539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1152F8A9-2EA7-4D93-82B2-39E4F5D7E4B4}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-17640" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1478,7 +1478,7 @@
   <autoFilter ref="A1:H228" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}">
     <filterColumn colId="1">
       <filters>
-        <filter val="FİZ 168"/>
+        <filter val="FİZ 174"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -1782,17 +1782,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H228"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="22.1796875" customWidth="1"/>
-    <col min="2" max="2" width="16.26953125" customWidth="1"/>
-    <col min="3" max="3" width="37.453125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="16.6328125" customWidth="1"/>
-    <col min="7" max="7" width="14.1796875" customWidth="1"/>
+    <col min="1" max="1" width="22.19921875" customWidth="1"/>
+    <col min="2" max="2" width="16.265625" customWidth="1"/>
+    <col min="3" max="3" width="37.46484375" customWidth="1"/>
+    <col min="5" max="5" width="10.265625" customWidth="1"/>
+    <col min="6" max="6" width="16.59765625" customWidth="1"/>
+    <col min="7" max="7" width="14.19921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1818,7 +1818,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -1844,7 +1844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -1870,7 +1870,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -1922,7 +1922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -1974,7 +1974,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2" t="s">
         <v>24</v>
       </c>
@@ -2000,7 +2000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -2052,7 +2052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
@@ -2130,7 +2130,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
@@ -2156,7 +2156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
         <v>21</v>
       </c>
@@ -2182,7 +2182,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
         <v>21</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
         <v>27</v>
       </c>
@@ -2260,7 +2260,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>24</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
         <v>21</v>
       </c>
@@ -2312,7 +2312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
         <v>24</v>
       </c>
@@ -2338,7 +2338,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
         <v>24</v>
       </c>
@@ -2364,7 +2364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>14</v>
       </c>
@@ -2416,7 +2416,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
         <v>17</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
         <v>19</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
         <v>21</v>
       </c>
@@ -2520,7 +2520,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
         <v>17</v>
       </c>
@@ -2546,7 +2546,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
         <v>27</v>
       </c>
@@ -2572,7 +2572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
         <v>19</v>
       </c>
@@ -2598,7 +2598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
         <v>27</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
         <v>21</v>
       </c>
@@ -2650,7 +2650,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
         <v>19</v>
       </c>
@@ -2676,7 +2676,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
         <v>21</v>
       </c>
@@ -2702,7 +2702,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
         <v>17</v>
       </c>
@@ -2728,7 +2728,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
         <v>7</v>
       </c>
@@ -2754,7 +2754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
         <v>7</v>
       </c>
@@ -2780,7 +2780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2" t="s">
         <v>27</v>
       </c>
@@ -2806,7 +2806,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
         <v>7</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
         <v>7</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
         <v>7</v>
       </c>
@@ -2884,7 +2884,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
         <v>21</v>
       </c>
@@ -2910,7 +2910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
         <v>14</v>
       </c>
@@ -2936,7 +2936,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
         <v>27</v>
       </c>
@@ -2962,7 +2962,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
         <v>27</v>
       </c>
@@ -2988,7 +2988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
         <v>7</v>
       </c>
@@ -3014,7 +3014,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
         <v>24</v>
       </c>
@@ -3040,7 +3040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
         <v>27</v>
       </c>
@@ -3066,7 +3066,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A50" s="2" t="s">
         <v>7</v>
       </c>
@@ -3092,7 +3092,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
         <v>21</v>
       </c>
@@ -3118,7 +3118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
         <v>21</v>
       </c>
@@ -3144,7 +3144,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
         <v>24</v>
       </c>
@@ -3170,7 +3170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
         <v>7</v>
       </c>
@@ -3196,7 +3196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
         <v>24</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A56" s="2" t="s">
         <v>14</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A57" s="2" t="s">
         <v>19</v>
       </c>
@@ -3274,7 +3274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
         <v>21</v>
       </c>
@@ -3300,7 +3300,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
         <v>21</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
         <v>21</v>
       </c>
@@ -3352,7 +3352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
         <v>21</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
         <v>21</v>
       </c>
@@ -3404,7 +3404,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
         <v>24</v>
       </c>
@@ -3430,7 +3430,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
         <v>21</v>
       </c>
@@ -3456,7 +3456,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A65" s="2" t="s">
         <v>27</v>
       </c>
@@ -3482,7 +3482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A66" s="2" t="s">
         <v>14</v>
       </c>
@@ -3508,7 +3508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A67" s="2" t="s">
         <v>19</v>
       </c>
@@ -3534,7 +3534,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A68" s="2" t="s">
         <v>24</v>
       </c>
@@ -3560,7 +3560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A69" s="2" t="s">
         <v>21</v>
       </c>
@@ -3586,7 +3586,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A70" s="2" t="s">
         <v>21</v>
       </c>
@@ -3612,7 +3612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A71" s="2" t="s">
         <v>7</v>
       </c>
@@ -3638,7 +3638,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A72" s="2" t="s">
         <v>24</v>
       </c>
@@ -3664,7 +3664,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A73" s="2" t="s">
         <v>27</v>
       </c>
@@ -3690,7 +3690,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A74" s="2" t="s">
         <v>19</v>
       </c>
@@ -3716,7 +3716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A75" s="2" t="s">
         <v>24</v>
       </c>
@@ -3742,7 +3742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A76" s="2" t="s">
         <v>14</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A77" s="2" t="s">
         <v>17</v>
       </c>
@@ -3794,7 +3794,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A78" s="2" t="s">
         <v>24</v>
       </c>
@@ -3820,7 +3820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A79" s="2" t="s">
         <v>19</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A80" s="2" t="s">
         <v>21</v>
       </c>
@@ -3872,7 +3872,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A81" s="2" t="s">
         <v>27</v>
       </c>
@@ -3898,7 +3898,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A82" s="2" t="s">
         <v>17</v>
       </c>
@@ -3924,7 +3924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A83" s="2" t="s">
         <v>19</v>
       </c>
@@ -3950,7 +3950,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A84" s="2" t="s">
         <v>19</v>
       </c>
@@ -3976,7 +3976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A85" s="2" t="s">
         <v>19</v>
       </c>
@@ -4002,7 +4002,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A86" s="2" t="s">
         <v>19</v>
       </c>
@@ -4028,7 +4028,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A87" s="2" t="s">
         <v>19</v>
       </c>
@@ -4054,7 +4054,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A88" s="2" t="s">
         <v>19</v>
       </c>
@@ -4080,7 +4080,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A89" s="2" t="s">
         <v>19</v>
       </c>
@@ -4106,7 +4106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A90" s="2" t="s">
         <v>19</v>
       </c>
@@ -4132,7 +4132,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A91" s="2" t="s">
         <v>19</v>
       </c>
@@ -4158,7 +4158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A92" s="2" t="s">
         <v>19</v>
       </c>
@@ -4184,7 +4184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A93" s="2" t="s">
         <v>14</v>
       </c>
@@ -4210,7 +4210,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A94" s="2" t="s">
         <v>21</v>
       </c>
@@ -4236,7 +4236,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A95" s="2" t="s">
         <v>24</v>
       </c>
@@ -4262,7 +4262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A96" s="2" t="s">
         <v>24</v>
       </c>
@@ -4288,7 +4288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A97" s="2" t="s">
         <v>17</v>
       </c>
@@ -4314,7 +4314,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A98" s="2" t="s">
         <v>27</v>
       </c>
@@ -4340,7 +4340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A99" s="2" t="s">
         <v>24</v>
       </c>
@@ -4366,7 +4366,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A100" s="2" t="s">
         <v>14</v>
       </c>
@@ -4392,7 +4392,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A101" s="2" t="s">
         <v>27</v>
       </c>
@@ -4418,7 +4418,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A102" s="2" t="s">
         <v>7</v>
       </c>
@@ -4444,7 +4444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A103" s="2" t="s">
         <v>7</v>
       </c>
@@ -4470,7 +4470,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A104" s="2" t="s">
         <v>7</v>
       </c>
@@ -4496,7 +4496,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A105" s="2" t="s">
         <v>7</v>
       </c>
@@ -4522,7 +4522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A106" s="2" t="s">
         <v>7</v>
       </c>
@@ -4548,7 +4548,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A107" s="2" t="s">
         <v>7</v>
       </c>
@@ -4574,7 +4574,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A108" s="2" t="s">
         <v>21</v>
       </c>
@@ -4600,7 +4600,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A109" s="2" t="s">
         <v>21</v>
       </c>
@@ -4626,7 +4626,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A110" s="2" t="s">
         <v>21</v>
       </c>
@@ -4652,7 +4652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A111" s="2" t="s">
         <v>24</v>
       </c>
@@ -4678,7 +4678,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A112" s="2" t="s">
         <v>24</v>
       </c>
@@ -4704,7 +4704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A113" s="2" t="s">
         <v>7</v>
       </c>
@@ -4730,7 +4730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A114" s="2" t="s">
         <v>24</v>
       </c>
@@ -4756,7 +4756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A115" s="2" t="s">
         <v>14</v>
       </c>
@@ -4782,7 +4782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A116" s="2" t="s">
         <v>19</v>
       </c>
@@ -4808,7 +4808,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A117" s="2" t="s">
         <v>14</v>
       </c>
@@ -4834,7 +4834,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A118" s="2" t="s">
         <v>27</v>
       </c>
@@ -4860,7 +4860,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A119" s="2" t="s">
         <v>24</v>
       </c>
@@ -4886,7 +4886,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A120" s="2" t="s">
         <v>24</v>
       </c>
@@ -4912,7 +4912,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A121" s="2" t="s">
         <v>17</v>
       </c>
@@ -4938,7 +4938,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A122" s="2" t="s">
         <v>17</v>
       </c>
@@ -4964,7 +4964,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A123" s="2" t="s">
         <v>17</v>
       </c>
@@ -4990,7 +4990,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A124" s="2" t="s">
         <v>19</v>
       </c>
@@ -5016,7 +5016,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A125" s="2" t="s">
         <v>7</v>
       </c>
@@ -5042,7 +5042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A126" s="2" t="s">
         <v>14</v>
       </c>
@@ -5068,7 +5068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A127" s="2" t="s">
         <v>27</v>
       </c>
@@ -5094,7 +5094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A128" s="2" t="s">
         <v>19</v>
       </c>
@@ -5120,7 +5120,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A129" s="2" t="s">
         <v>24</v>
       </c>
@@ -5146,7 +5146,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A130" s="2" t="s">
         <v>17</v>
       </c>
@@ -5172,7 +5172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A131" s="2" t="s">
         <v>14</v>
       </c>
@@ -5198,7 +5198,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A132" s="2" t="s">
         <v>7</v>
       </c>
@@ -5224,7 +5224,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A133" s="2" t="s">
         <v>21</v>
       </c>
@@ -5250,7 +5250,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A134" s="2" t="s">
         <v>14</v>
       </c>
@@ -5276,7 +5276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A135" s="2" t="s">
         <v>24</v>
       </c>
@@ -5302,7 +5302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A136" s="2" t="s">
         <v>17</v>
       </c>
@@ -5328,7 +5328,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A137" s="2" t="s">
         <v>17</v>
       </c>
@@ -5354,7 +5354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A138" s="2" t="s">
         <v>24</v>
       </c>
@@ -5380,7 +5380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A139" s="2" t="s">
         <v>24</v>
       </c>
@@ -5406,7 +5406,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A140" s="2" t="s">
         <v>14</v>
       </c>
@@ -5432,7 +5432,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A141" s="2" t="s">
         <v>17</v>
       </c>
@@ -5458,7 +5458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A142" s="2" t="s">
         <v>24</v>
       </c>
@@ -5484,7 +5484,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A143" s="2" t="s">
         <v>19</v>
       </c>
@@ -5510,7 +5510,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A144" s="2" t="s">
         <v>7</v>
       </c>
@@ -5536,7 +5536,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A145" s="2" t="s">
         <v>27</v>
       </c>
@@ -5562,7 +5562,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A146" s="2" t="s">
         <v>21</v>
       </c>
@@ -5588,7 +5588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A147" s="2" t="s">
         <v>24</v>
       </c>
@@ -5614,7 +5614,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A148" s="2" t="s">
         <v>17</v>
       </c>
@@ -5640,7 +5640,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A149" s="2" t="s">
         <v>7</v>
       </c>
@@ -5666,7 +5666,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A150" s="2" t="s">
         <v>21</v>
       </c>
@@ -5692,7 +5692,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A151" s="2" t="s">
         <v>21</v>
       </c>
@@ -5718,7 +5718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A152" s="2" t="s">
         <v>14</v>
       </c>
@@ -5744,7 +5744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A153" s="2" t="s">
         <v>17</v>
       </c>
@@ -5770,7 +5770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A154" s="2" t="s">
         <v>7</v>
       </c>
@@ -5796,7 +5796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A155" s="2" t="s">
         <v>19</v>
       </c>
@@ -5822,7 +5822,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A156" s="2" t="s">
         <v>14</v>
       </c>
@@ -5848,7 +5848,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A157" s="2" t="s">
         <v>24</v>
       </c>
@@ -5874,7 +5874,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A158" s="2" t="s">
         <v>24</v>
       </c>
@@ -5900,7 +5900,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A159" s="2" t="s">
         <v>24</v>
       </c>
@@ -5926,7 +5926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A160" s="2" t="s">
         <v>14</v>
       </c>
@@ -5952,7 +5952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A161" s="2" t="s">
         <v>14</v>
       </c>
@@ -5978,7 +5978,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A162" s="2" t="s">
         <v>27</v>
       </c>
@@ -6004,7 +6004,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A163" s="2" t="s">
         <v>17</v>
       </c>
@@ -6030,7 +6030,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A164" s="2" t="s">
         <v>19</v>
       </c>
@@ -6056,7 +6056,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A165" s="2" t="s">
         <v>21</v>
       </c>
@@ -6082,7 +6082,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A166" s="2" t="s">
         <v>19</v>
       </c>
@@ -6108,7 +6108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A167" s="2" t="s">
         <v>7</v>
       </c>
@@ -6134,7 +6134,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A168" s="2" t="s">
         <v>19</v>
       </c>
@@ -6160,7 +6160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A169" s="2" t="s">
         <v>7</v>
       </c>
@@ -6186,7 +6186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A170" s="2" t="s">
         <v>27</v>
       </c>
@@ -6212,7 +6212,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A171" s="2" t="s">
         <v>21</v>
       </c>
@@ -6238,7 +6238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A172" s="2" t="s">
         <v>7</v>
       </c>
@@ -6264,7 +6264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A173" s="2" t="s">
         <v>21</v>
       </c>
@@ -6290,7 +6290,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A174" s="2" t="s">
         <v>21</v>
       </c>
@@ -6316,7 +6316,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A175" s="2" t="s">
         <v>21</v>
       </c>
@@ -6342,7 +6342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A176" s="2" t="s">
         <v>21</v>
       </c>
@@ -6368,7 +6368,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A177" s="2" t="s">
         <v>21</v>
       </c>
@@ -6394,7 +6394,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A178" s="2" t="s">
         <v>7</v>
       </c>
@@ -6420,7 +6420,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A179" s="2" t="s">
         <v>19</v>
       </c>
@@ -6446,7 +6446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A180" s="2" t="s">
         <v>21</v>
       </c>
@@ -6472,7 +6472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A181" s="2" t="s">
         <v>19</v>
       </c>
@@ -6498,7 +6498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A182" s="2" t="s">
         <v>24</v>
       </c>
@@ -6524,7 +6524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A183" s="2" t="s">
         <v>17</v>
       </c>
@@ -6550,7 +6550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A184" s="2" t="s">
         <v>24</v>
       </c>
@@ -6576,7 +6576,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A185" s="2" t="s">
         <v>27</v>
       </c>
@@ -6602,7 +6602,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A186" s="2" t="s">
         <v>17</v>
       </c>
@@ -6628,7 +6628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A187" s="2" t="s">
         <v>21</v>
       </c>
@@ -6654,7 +6654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A188" s="2" t="s">
         <v>7</v>
       </c>
@@ -6680,7 +6680,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A189" s="2" t="s">
         <v>21</v>
       </c>
@@ -6706,7 +6706,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A190" s="2" t="s">
         <v>7</v>
       </c>
@@ -6732,7 +6732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A191" s="2" t="s">
         <v>24</v>
       </c>
@@ -6758,7 +6758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A192" s="2" t="s">
         <v>7</v>
       </c>
@@ -6784,7 +6784,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A193" s="2" t="s">
         <v>7</v>
       </c>
@@ -6810,7 +6810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A194" s="2" t="s">
         <v>19</v>
       </c>
@@ -6836,7 +6836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A195" s="2" t="s">
         <v>14</v>
       </c>
@@ -6862,7 +6862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A196" s="2" t="s">
         <v>24</v>
       </c>
@@ -6888,7 +6888,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A197" s="2" t="s">
         <v>14</v>
       </c>
@@ -6914,7 +6914,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A198" s="2" t="s">
         <v>24</v>
       </c>
@@ -6940,7 +6940,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A199" s="2" t="s">
         <v>27</v>
       </c>
@@ -6966,7 +6966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A200" s="2" t="s">
         <v>17</v>
       </c>
@@ -6992,7 +6992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A201" s="2" t="s">
         <v>14</v>
       </c>
@@ -7018,7 +7018,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A202" s="2" t="s">
         <v>14</v>
       </c>
@@ -7044,7 +7044,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A203" s="2" t="s">
         <v>19</v>
       </c>
@@ -7070,7 +7070,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A204" s="2" t="s">
         <v>24</v>
       </c>
@@ -7096,7 +7096,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A205" s="2" t="s">
         <v>27</v>
       </c>
@@ -7122,7 +7122,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A206" s="2" t="s">
         <v>24</v>
       </c>
@@ -7148,7 +7148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A207" s="2" t="s">
         <v>19</v>
       </c>
@@ -7174,7 +7174,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A208" s="2" t="s">
         <v>14</v>
       </c>
@@ -7200,7 +7200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A209" s="2" t="s">
         <v>19</v>
       </c>
@@ -7226,7 +7226,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A210" s="2" t="s">
         <v>27</v>
       </c>
@@ -7252,7 +7252,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A211" s="2" t="s">
         <v>19</v>
       </c>
@@ -7278,7 +7278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A212" s="2" t="s">
         <v>24</v>
       </c>
@@ -7304,7 +7304,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A213" s="2" t="s">
         <v>14</v>
       </c>
@@ -7330,7 +7330,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A214" s="2" t="s">
         <v>14</v>
       </c>
@@ -7356,7 +7356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A215" s="2" t="s">
         <v>17</v>
       </c>
@@ -7382,7 +7382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A216" s="2" t="s">
         <v>19</v>
       </c>
@@ -7408,7 +7408,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A217" s="2" t="s">
         <v>21</v>
       </c>
@@ -7434,7 +7434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A218" s="2" t="s">
         <v>14</v>
       </c>
@@ -7460,7 +7460,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A219" s="2" t="s">
         <v>27</v>
       </c>
@@ -7486,7 +7486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A220" s="2" t="s">
         <v>19</v>
       </c>
@@ -7512,7 +7512,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A221" s="2" t="s">
         <v>24</v>
       </c>
@@ -7538,7 +7538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A222" s="2" t="s">
         <v>14</v>
       </c>
@@ -7564,7 +7564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A223" s="2" t="s">
         <v>14</v>
       </c>
@@ -7590,7 +7590,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A224" s="2" t="s">
         <v>14</v>
       </c>
@@ -7616,7 +7616,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A225" s="2" t="s">
         <v>17</v>
       </c>
@@ -7642,7 +7642,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A226" s="2" t="s">
         <v>14</v>
       </c>
@@ -7668,7 +7668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A227" s="2" t="s">
         <v>17</v>
       </c>
@@ -7694,7 +7694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="228" spans="1:8" hidden="1" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A228" s="2" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
manuel fac wise done. TODO: Analysis
</commit_message>
<xml_diff>
--- a/data/BerkData2.xlsx
+++ b/data/BerkData2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e402f802124af4b/Masaüstü/Projects/Campus-Scheduling/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{2C943E96-C6E4-40C4-888D-FAADD3A22539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1152F8A9-2EA7-4D93-82B2-39E4F5D7E4B4}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{2C943E96-C6E4-40C4-888D-FAADD3A22539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73EF178F-B942-4E9E-B37E-B80A3349A76A}"/>
   <bookViews>
     <workbookView xWindow="-17640" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="433">
   <si>
     <t>DepartmentName</t>
   </si>
@@ -1100,12 +1100,6 @@
   </si>
   <si>
     <t>Seminar</t>
-  </si>
-  <si>
-    <t>MAK 314</t>
-  </si>
-  <si>
-    <t>Seminer</t>
   </si>
   <si>
     <t>CSE 474</t>
@@ -1473,15 +1467,24 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}" name="Table1" displayName="Table1" ref="A1:H228" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
-  <autoFilter ref="A1:H228" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}" name="Table1" displayName="Table1" ref="A1:H227" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
+  <autoFilter ref="A1:H227" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}">
     <filterColumn colId="1">
       <filters>
+        <filter val="EEM 370"/>
         <filter val="FİZ 174"/>
+        <filter val="GIDA 324"/>
       </filters>
     </filterColumn>
   </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A8:H220">
+    <sortCondition ref="B1:B227"/>
+  </sortState>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{E28ED7F9-92E9-43FB-898A-30B6DDD841D3}" name="DepartmentName" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{A24A0F99-F460-4F6A-BEC2-81C68341B7ED}" name="CourseCode" dataDxfId="6"/>
@@ -1781,7 +1784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H228"/>
+  <dimension ref="A1:H227"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="22.19921875" customWidth="1"/>
@@ -1815,7 +1818,7 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
     </row>
     <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
@@ -1979,25 +1982,25 @@
         <v>24</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="D8" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F8" s="2">
-        <v>1502554</v>
+        <v>3952988</v>
       </c>
       <c r="G8" s="2">
-        <v>18</v>
+        <v>180</v>
       </c>
       <c r="H8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
@@ -2156,7 +2159,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
         <v>21</v>
       </c>
@@ -2265,25 +2268,25 @@
         <v>24</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>48</v>
+        <v>372</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>49</v>
+        <v>371</v>
       </c>
       <c r="D19" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F19" s="2">
-        <v>2579557</v>
+        <v>2554019</v>
       </c>
       <c r="G19" s="2">
-        <v>16</v>
+        <v>141</v>
       </c>
       <c r="H19" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
@@ -2317,10 +2320,10 @@
         <v>24</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D21" s="2">
         <v>1</v>
@@ -2329,13 +2332,13 @@
         <v>10</v>
       </c>
       <c r="F21" s="2">
-        <v>3952988</v>
+        <v>1307360</v>
       </c>
       <c r="G21" s="2">
-        <v>180</v>
+        <v>115</v>
       </c>
       <c r="H21" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
@@ -2343,25 +2346,25 @@
         <v>24</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>54</v>
+        <v>162</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>55</v>
+        <v>161</v>
       </c>
       <c r="D22" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F22" s="2">
-        <v>6112322</v>
+        <v>2132049</v>
       </c>
       <c r="G22" s="2">
-        <v>24</v>
+        <v>123</v>
       </c>
       <c r="H22" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
@@ -2421,10 +2424,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>60</v>
+        <v>265</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>59</v>
+        <v>264</v>
       </c>
       <c r="D25" s="2">
         <v>1</v>
@@ -2433,10 +2436,10 @@
         <v>10</v>
       </c>
       <c r="F25" s="2">
-        <v>1307360</v>
+        <v>1041914</v>
       </c>
       <c r="G25" s="2">
-        <v>115</v>
+        <v>160</v>
       </c>
       <c r="H25" s="2">
         <v>0</v>
@@ -3019,22 +3022,22 @@
         <v>24</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>103</v>
+        <v>301</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>104</v>
+        <v>302</v>
       </c>
       <c r="D48" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F48" s="2">
-        <v>1494406</v>
+        <v>1235319</v>
       </c>
       <c r="G48" s="2">
-        <v>18</v>
+        <v>99</v>
       </c>
       <c r="H48" s="2">
         <v>0</v>
@@ -3149,10 +3152,10 @@
         <v>24</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>113</v>
+        <v>299</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>114</v>
+        <v>300</v>
       </c>
       <c r="D53" s="2">
         <v>2</v>
@@ -3164,7 +3167,7 @@
         <v>1618088</v>
       </c>
       <c r="G53" s="2">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="H53" s="2">
         <v>0</v>
@@ -3201,22 +3204,22 @@
         <v>24</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>117</v>
+        <v>398</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>118</v>
+        <v>399</v>
       </c>
       <c r="D55" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F55" s="2">
         <v>2994200</v>
       </c>
       <c r="G55" s="2">
-        <v>18</v>
+        <v>131</v>
       </c>
       <c r="H55" s="2">
         <v>0</v>
@@ -3409,10 +3412,10 @@
         <v>24</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>132</v>
+        <v>113</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>133</v>
+        <v>114</v>
       </c>
       <c r="D63" s="2">
         <v>2</v>
@@ -3421,10 +3424,10 @@
         <v>10</v>
       </c>
       <c r="F63" s="2">
-        <v>1600939</v>
+        <v>1618088</v>
       </c>
       <c r="G63" s="2">
-        <v>80</v>
+        <v>96</v>
       </c>
       <c r="H63" s="2">
         <v>0</v>
@@ -3539,22 +3542,22 @@
         <v>24</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>142</v>
+        <v>303</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>143</v>
+        <v>304</v>
       </c>
       <c r="D68" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F68" s="2">
-        <v>1502554</v>
+        <v>2832797</v>
       </c>
       <c r="G68" s="2">
-        <v>16</v>
+        <v>97</v>
       </c>
       <c r="H68" s="2">
         <v>0</v>
@@ -3643,22 +3646,22 @@
         <v>24</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>150</v>
+        <v>132</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>151</v>
+        <v>133</v>
       </c>
       <c r="D72" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F72" s="2">
-        <v>5018255</v>
+        <v>1600939</v>
       </c>
       <c r="G72" s="2">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="H72" s="2">
         <v>0</v>
@@ -3721,22 +3724,22 @@
         <v>24</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>156</v>
+        <v>272</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>157</v>
+        <v>273</v>
       </c>
       <c r="D75" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F75" s="2">
-        <v>5018255</v>
+        <v>2579557</v>
       </c>
       <c r="G75" s="2">
-        <v>19</v>
+        <v>117</v>
       </c>
       <c r="H75" s="2">
         <v>0</v>
@@ -3799,22 +3802,22 @@
         <v>24</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>162</v>
+        <v>230</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>161</v>
+        <v>231</v>
       </c>
       <c r="D78" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F78" s="2">
-        <v>2132049</v>
+        <v>3952988</v>
       </c>
       <c r="G78" s="2">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="H78" s="2">
         <v>0</v>
@@ -4132,7 +4135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A91" s="2" t="s">
         <v>19</v>
       </c>
@@ -4241,22 +4244,22 @@
         <v>24</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>192</v>
+        <v>270</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>193</v>
+        <v>271</v>
       </c>
       <c r="D95" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F95" s="2">
-        <v>2576518</v>
+        <v>1457877</v>
       </c>
       <c r="G95" s="2">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="H95" s="2">
         <v>0</v>
@@ -4267,22 +4270,22 @@
         <v>24</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="D96" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F96" s="2">
-        <v>1210302</v>
+        <v>5299061</v>
       </c>
       <c r="G96" s="2">
-        <v>34</v>
+        <v>83</v>
       </c>
       <c r="H96" s="2">
         <v>0</v>
@@ -4345,10 +4348,10 @@
         <v>24</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>200</v>
+        <v>226</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>201</v>
+        <v>227</v>
       </c>
       <c r="D99" s="2">
         <v>3</v>
@@ -4357,10 +4360,10 @@
         <v>10</v>
       </c>
       <c r="F99" s="2">
-        <v>5299061</v>
+        <v>2576518</v>
       </c>
       <c r="G99" s="2">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="H99" s="2">
         <v>0</v>
@@ -4657,22 +4660,22 @@
         <v>24</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>224</v>
+        <v>368</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>225</v>
+        <v>369</v>
       </c>
       <c r="D111" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F111" s="2">
-        <v>5299061</v>
+        <v>1707115</v>
       </c>
       <c r="G111" s="2">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H111" s="2">
         <v>0</v>
@@ -4680,13 +4683,13 @@
     </row>
     <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A112" s="2" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D112" s="2">
         <v>3</v>
@@ -4695,10 +4698,10 @@
         <v>10</v>
       </c>
       <c r="F112" s="2">
-        <v>2576518</v>
+        <v>1842843</v>
       </c>
       <c r="G112" s="2">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="H112" s="2">
         <v>0</v>
@@ -4706,25 +4709,25 @@
     </row>
     <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A113" s="2" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>228</v>
+        <v>387</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>229</v>
+        <v>388</v>
       </c>
       <c r="D113" s="2">
         <v>3</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F113" s="2">
-        <v>1842843</v>
+        <v>1235319</v>
       </c>
       <c r="G113" s="2">
-        <v>74</v>
+        <v>21</v>
       </c>
       <c r="H113" s="2">
         <v>0</v>
@@ -4732,25 +4735,25 @@
     </row>
     <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A114" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D114" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E114" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F114" s="2">
-        <v>3952988</v>
+        <v>2977082</v>
       </c>
       <c r="G114" s="2">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="H114" s="2">
         <v>0</v>
@@ -4758,25 +4761,25 @@
     </row>
     <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A115" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D115" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F115" s="2">
-        <v>2977082</v>
+        <v>3258742</v>
       </c>
       <c r="G115" s="2">
-        <v>120</v>
+        <v>48</v>
       </c>
       <c r="H115" s="2">
         <v>0</v>
@@ -4784,25 +4787,25 @@
     </row>
     <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A116" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D116" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F116" s="2">
-        <v>3258742</v>
+        <v>6933704</v>
       </c>
       <c r="G116" s="2">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H116" s="2">
         <v>0</v>
@@ -4810,25 +4813,25 @@
     </row>
     <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A117" s="2" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C117" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D117" s="2">
         <v>4</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F117" s="2">
-        <v>6933704</v>
+        <v>2355205</v>
       </c>
       <c r="G117" s="2">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="H117" s="2">
         <v>0</v>
@@ -4836,25 +4839,25 @@
     </row>
     <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A118" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="C118" s="2" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="D118" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F118" s="2">
-        <v>2355205</v>
+        <v>4576344</v>
       </c>
       <c r="G118" s="2">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="H118" s="2">
         <v>0</v>
@@ -4888,25 +4891,25 @@
     </row>
     <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A120" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D120" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F120" s="2">
-        <v>4576344</v>
+        <v>1410757</v>
       </c>
       <c r="G120" s="2">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H120" s="2">
         <v>0</v>
@@ -4917,22 +4920,22 @@
         <v>17</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D121" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F121" s="2">
-        <v>1410757</v>
+        <v>2446060</v>
       </c>
       <c r="G121" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H121" s="2">
         <v>0</v>
@@ -4943,10 +4946,10 @@
         <v>17</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D122" s="2">
         <v>3</v>
@@ -4955,7 +4958,7 @@
         <v>13</v>
       </c>
       <c r="F122" s="2">
-        <v>2446060</v>
+        <v>1608770</v>
       </c>
       <c r="G122" s="2">
         <v>5</v>
@@ -4966,25 +4969,25 @@
     </row>
     <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A123" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D123" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E123" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F123" s="2">
-        <v>1608770</v>
+        <v>2571190</v>
       </c>
       <c r="G123" s="2">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="H123" s="2">
         <v>0</v>
@@ -4992,33 +4995,33 @@
     </row>
     <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A124" s="2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C124" s="2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D124" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F124" s="2">
-        <v>2571190</v>
+        <v>1267061</v>
       </c>
       <c r="G124" s="2">
-        <v>45</v>
+        <v>115</v>
       </c>
       <c r="H124" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A125" s="2" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B125" s="2" t="s">
         <v>251</v>
@@ -5033,18 +5036,18 @@
         <v>10</v>
       </c>
       <c r="F125" s="2">
-        <v>1267061</v>
+        <v>3074554</v>
       </c>
       <c r="G125" s="2">
-        <v>115</v>
+        <v>73</v>
       </c>
       <c r="H125" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A126" s="2" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B126" s="2" t="s">
         <v>251</v>
@@ -5062,7 +5065,7 @@
         <v>3074554</v>
       </c>
       <c r="G126" s="2">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="H126" s="2">
         <v>0</v>
@@ -5070,7 +5073,7 @@
     </row>
     <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A127" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B127" s="2" t="s">
         <v>251</v>
@@ -5085,10 +5088,10 @@
         <v>10</v>
       </c>
       <c r="F127" s="2">
-        <v>3074554</v>
+        <v>2571190</v>
       </c>
       <c r="G127" s="2">
-        <v>18</v>
+        <v>54</v>
       </c>
       <c r="H127" s="2">
         <v>0</v>
@@ -5096,25 +5099,25 @@
     </row>
     <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A128" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>251</v>
+        <v>103</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>252</v>
+        <v>104</v>
       </c>
       <c r="D128" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F128" s="2">
-        <v>2571190</v>
+        <v>1494406</v>
       </c>
       <c r="G128" s="2">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="H128" s="2">
         <v>0</v>
@@ -5122,25 +5125,25 @@
     </row>
     <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A129" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D129" s="2">
         <v>4</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F129" s="2">
-        <v>1618088</v>
+        <v>1608770</v>
       </c>
       <c r="G129" s="2">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="H129" s="2">
         <v>0</v>
@@ -5148,25 +5151,25 @@
     </row>
     <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A130" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D130" s="2">
         <v>4</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F130" s="2">
-        <v>1608770</v>
+        <v>2587917</v>
       </c>
       <c r="G130" s="2">
-        <v>9</v>
+        <v>20</v>
       </c>
       <c r="H130" s="2">
         <v>0</v>
@@ -5174,25 +5177,25 @@
     </row>
     <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A131" s="2" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D131" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F131" s="2">
-        <v>2587917</v>
+        <v>4693090</v>
       </c>
       <c r="G131" s="2">
-        <v>20</v>
+        <v>135</v>
       </c>
       <c r="H131" s="2">
         <v>0</v>
@@ -5200,16 +5203,16 @@
     </row>
     <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A132" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C132" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D132" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>10</v>
@@ -5218,7 +5221,7 @@
         <v>4693090</v>
       </c>
       <c r="G132" s="2">
-        <v>135</v>
+        <v>203</v>
       </c>
       <c r="H132" s="2">
         <v>0</v>
@@ -5226,13 +5229,13 @@
     </row>
     <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A133" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D133" s="2">
         <v>1</v>
@@ -5241,10 +5244,10 @@
         <v>10</v>
       </c>
       <c r="F133" s="2">
-        <v>4693090</v>
+        <v>1041914</v>
       </c>
       <c r="G133" s="2">
-        <v>203</v>
+        <v>110</v>
       </c>
       <c r="H133" s="2">
         <v>0</v>
@@ -5252,51 +5255,51 @@
     </row>
     <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A134" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>263</v>
+        <v>48</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>264</v>
+        <v>49</v>
       </c>
       <c r="D134" s="2">
+        <v>4</v>
+      </c>
+      <c r="E134" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F134" s="2">
+        <v>2579557</v>
+      </c>
+      <c r="G134" s="2">
+        <v>16</v>
+      </c>
+      <c r="H134" s="2">
         <v>1</v>
-      </c>
-      <c r="E134" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F134" s="2">
-        <v>1041914</v>
-      </c>
-      <c r="G134" s="2">
-        <v>110</v>
-      </c>
-      <c r="H134" s="2">
-        <v>0</v>
       </c>
     </row>
     <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A135" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D135" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F135" s="2">
-        <v>1041914</v>
+        <v>3258742</v>
       </c>
       <c r="G135" s="2">
-        <v>160</v>
+        <v>9</v>
       </c>
       <c r="H135" s="2">
         <v>0</v>
@@ -5307,22 +5310,22 @@
         <v>17</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D136" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F136" s="2">
-        <v>3258742</v>
+        <v>3633158</v>
       </c>
       <c r="G136" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H136" s="2">
         <v>0</v>
@@ -5330,28 +5333,28 @@
     </row>
     <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A137" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>268</v>
+        <v>54</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>269</v>
+        <v>55</v>
       </c>
       <c r="D137" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E137" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F137" s="2">
-        <v>3633158</v>
+        <v>6112322</v>
       </c>
       <c r="G137" s="2">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="H137" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
@@ -5359,22 +5362,22 @@
         <v>24</v>
       </c>
       <c r="B138" s="2" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="D138" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E138" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F138" s="2">
-        <v>1457877</v>
+        <v>1618088</v>
       </c>
       <c r="G138" s="2">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="H138" s="2">
         <v>0</v>
@@ -5382,25 +5385,25 @@
     </row>
     <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A139" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B139" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C139" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D139" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F139" s="2">
-        <v>2579557</v>
+        <v>2550816</v>
       </c>
       <c r="G139" s="2">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="H139" s="2">
         <v>0</v>
@@ -5408,7 +5411,7 @@
     </row>
     <row r="140" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A140" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>274</v>
@@ -5426,7 +5429,7 @@
         <v>2550816</v>
       </c>
       <c r="G140" s="2">
-        <v>102</v>
+        <v>15</v>
       </c>
       <c r="H140" s="2">
         <v>0</v>
@@ -5434,25 +5437,25 @@
     </row>
     <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A141" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B141" s="2" t="s">
-        <v>274</v>
+        <v>383</v>
       </c>
       <c r="C141" s="2" t="s">
-        <v>275</v>
+        <v>384</v>
       </c>
       <c r="D141" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F141" s="2">
-        <v>2550816</v>
+        <v>1235319</v>
       </c>
       <c r="G141" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H141" s="2">
         <v>0</v>
@@ -5460,7 +5463,7 @@
     </row>
     <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A142" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B142" s="2" t="s">
         <v>274</v>
@@ -5475,10 +5478,10 @@
         <v>10</v>
       </c>
       <c r="F142" s="2">
-        <v>1739868</v>
+        <v>4117613</v>
       </c>
       <c r="G142" s="2">
-        <v>159</v>
+        <v>99</v>
       </c>
       <c r="H142" s="2">
         <v>0</v>
@@ -5486,13 +5489,13 @@
     </row>
     <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A143" s="2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B143" s="2" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="C143" s="2" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="D143" s="2">
         <v>1</v>
@@ -5501,10 +5504,10 @@
         <v>10</v>
       </c>
       <c r="F143" s="2">
-        <v>4117613</v>
+        <v>4828331</v>
       </c>
       <c r="G143" s="2">
-        <v>99</v>
+        <v>160</v>
       </c>
       <c r="H143" s="2">
         <v>0</v>
@@ -5512,7 +5515,7 @@
     </row>
     <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A144" s="2" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B144" s="2" t="s">
         <v>277</v>
@@ -5527,10 +5530,10 @@
         <v>10</v>
       </c>
       <c r="F144" s="2">
-        <v>4828331</v>
+        <v>1875741</v>
       </c>
       <c r="G144" s="2">
-        <v>160</v>
+        <v>19</v>
       </c>
       <c r="H144" s="2">
         <v>0</v>
@@ -5538,7 +5541,7 @@
     </row>
     <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A145" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B145" s="2" t="s">
         <v>277</v>
@@ -5556,7 +5559,7 @@
         <v>1875741</v>
       </c>
       <c r="G145" s="2">
-        <v>19</v>
+        <v>189</v>
       </c>
       <c r="H145" s="2">
         <v>0</v>
@@ -5564,25 +5567,25 @@
     </row>
     <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A146" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B146" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C146" s="2" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D146" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E146" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F146" s="2">
-        <v>1875741</v>
+        <v>1457877</v>
       </c>
       <c r="G146" s="2">
-        <v>189</v>
+        <v>19</v>
       </c>
       <c r="H146" s="2">
         <v>0</v>
@@ -5590,25 +5593,25 @@
     </row>
     <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A147" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B147" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C147" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="D147" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E147" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F147" s="2">
-        <v>1457877</v>
+        <v>1009202</v>
       </c>
       <c r="G147" s="2">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="H147" s="2">
         <v>0</v>
@@ -5616,39 +5619,39 @@
     </row>
     <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A148" s="2" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B148" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C148" s="2" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="D148" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F148" s="2">
-        <v>1009202</v>
+        <v>1267061</v>
       </c>
       <c r="G148" s="2">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="H148" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A149" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B149" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C149" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D149" s="2">
         <v>4</v>
@@ -5657,13 +5660,13 @@
         <v>13</v>
       </c>
       <c r="F149" s="2">
-        <v>1267061</v>
+        <v>3041802</v>
       </c>
       <c r="G149" s="2">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="H149" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
@@ -5671,22 +5674,22 @@
         <v>21</v>
       </c>
       <c r="B150" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C150" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="D150" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E150" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F150" s="2">
-        <v>3041802</v>
+        <v>1121323</v>
       </c>
       <c r="G150" s="2">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="H150" s="2">
         <v>0</v>
@@ -5694,25 +5697,25 @@
     </row>
     <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A151" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B151" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C151" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="D151" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E151" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F151" s="2">
-        <v>1121323</v>
+        <v>2028216</v>
       </c>
       <c r="G151" s="2">
-        <v>45</v>
+        <v>24</v>
       </c>
       <c r="H151" s="2">
         <v>0</v>
@@ -5720,25 +5723,25 @@
     </row>
     <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A152" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B152" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C152" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D152" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E152" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F152" s="2">
-        <v>2028216</v>
+        <v>1009202</v>
       </c>
       <c r="G152" s="2">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H152" s="2">
         <v>0</v>
@@ -5746,25 +5749,25 @@
     </row>
     <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A153" s="2" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B153" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D153" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E153" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F153" s="2">
-        <v>1009202</v>
+        <v>3013005</v>
       </c>
       <c r="G153" s="2">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="H153" s="2">
         <v>0</v>
@@ -5772,25 +5775,25 @@
     </row>
     <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A154" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="B154" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D154" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E154" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F154" s="2">
-        <v>3013005</v>
+        <v>2311022</v>
       </c>
       <c r="G154" s="2">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="H154" s="2">
         <v>0</v>
@@ -5798,25 +5801,25 @@
     </row>
     <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A155" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B155" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C155" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D155" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F155" s="2">
-        <v>2311022</v>
+        <v>2391172</v>
       </c>
       <c r="G155" s="2">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="H155" s="2">
         <v>0</v>
@@ -5824,25 +5827,25 @@
     </row>
     <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A156" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B156" s="2" t="s">
-        <v>297</v>
+        <v>150</v>
       </c>
       <c r="C156" s="2" t="s">
-        <v>298</v>
+        <v>151</v>
       </c>
       <c r="D156" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E156" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F156" s="2">
-        <v>2391172</v>
+        <v>5018255</v>
       </c>
       <c r="G156" s="2">
-        <v>80</v>
+        <v>17</v>
       </c>
       <c r="H156" s="2">
         <v>0</v>
@@ -5853,22 +5856,22 @@
         <v>24</v>
       </c>
       <c r="B157" s="2" t="s">
-        <v>299</v>
+        <v>156</v>
       </c>
       <c r="C157" s="2" t="s">
-        <v>300</v>
+        <v>157</v>
       </c>
       <c r="D157" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E157" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F157" s="2">
-        <v>1618088</v>
+        <v>5018255</v>
       </c>
       <c r="G157" s="2">
-        <v>99</v>
+        <v>19</v>
       </c>
       <c r="H157" s="2">
         <v>0</v>
@@ -5879,22 +5882,22 @@
         <v>24</v>
       </c>
       <c r="B158" s="2" t="s">
-        <v>301</v>
+        <v>117</v>
       </c>
       <c r="C158" s="2" t="s">
-        <v>302</v>
+        <v>118</v>
       </c>
       <c r="D158" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E158" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F158" s="2">
-        <v>1235319</v>
+        <v>2994200</v>
       </c>
       <c r="G158" s="2">
-        <v>99</v>
+        <v>18</v>
       </c>
       <c r="H158" s="2">
         <v>0</v>
@@ -5902,25 +5905,25 @@
     </row>
     <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A159" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B159" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C159" s="2" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D159" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E159" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F159" s="2">
-        <v>2832797</v>
+        <v>3979315</v>
       </c>
       <c r="G159" s="2">
-        <v>97</v>
+        <v>20</v>
       </c>
       <c r="H159" s="2">
         <v>0</v>
@@ -5931,33 +5934,33 @@
         <v>14</v>
       </c>
       <c r="B160" s="2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C160" s="2" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D160" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E160" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F160" s="2">
-        <v>3979315</v>
+        <v>3258742</v>
       </c>
       <c r="G160" s="2">
-        <v>20</v>
+        <v>75</v>
       </c>
       <c r="H160" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A161" s="2" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B161" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C161" s="2" t="s">
         <v>308</v>
@@ -5966,39 +5969,39 @@
         <v>2</v>
       </c>
       <c r="E161" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F161" s="2">
-        <v>3258742</v>
+        <v>3070901</v>
       </c>
       <c r="G161" s="2">
-        <v>75</v>
+        <v>15</v>
       </c>
       <c r="H161" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A162" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B162" s="2" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C162" s="2" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D162" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E162" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F162" s="2">
-        <v>3070901</v>
+        <v>3633158</v>
       </c>
       <c r="G162" s="2">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="H162" s="2">
         <v>0</v>
@@ -6006,25 +6009,25 @@
     </row>
     <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A163" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B163" s="2" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="C163" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D163" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E163" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F163" s="2">
-        <v>3633158</v>
+        <v>3850625</v>
       </c>
       <c r="G163" s="2">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="H163" s="2">
         <v>0</v>
@@ -6032,25 +6035,25 @@
     </row>
     <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A164" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B164" s="2" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="C164" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D164" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E164" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F164" s="2">
-        <v>3850625</v>
+        <v>4721220</v>
       </c>
       <c r="G164" s="2">
-        <v>97</v>
+        <v>144</v>
       </c>
       <c r="H164" s="2">
         <v>0</v>
@@ -6058,25 +6061,25 @@
     </row>
     <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A165" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B165" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="C165" s="2" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="D165" s="2">
         <v>3</v>
       </c>
       <c r="E165" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F165" s="2">
-        <v>4721220</v>
+        <v>1093367</v>
       </c>
       <c r="G165" s="2">
-        <v>144</v>
+        <v>39</v>
       </c>
       <c r="H165" s="2">
         <v>0</v>
@@ -6084,25 +6087,25 @@
     </row>
     <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A166" s="2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B166" s="2" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C166" s="2" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="D166" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E166" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F166" s="2">
-        <v>1093367</v>
+        <v>2238227</v>
       </c>
       <c r="G166" s="2">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="H166" s="2">
         <v>0</v>
@@ -6110,13 +6113,13 @@
     </row>
     <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A167" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="B167" s="2" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="C167" s="2" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D167" s="2">
         <v>4</v>
@@ -6125,47 +6128,47 @@
         <v>13</v>
       </c>
       <c r="F167" s="2">
-        <v>2238227</v>
+        <v>1086552</v>
       </c>
       <c r="G167" s="2">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="H167" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A168" s="2" t="s">
-        <v>19</v>
+        <v>7</v>
       </c>
       <c r="B168" s="2" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="D168" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E168" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F168" s="2">
-        <v>1086552</v>
+        <v>5320332</v>
       </c>
       <c r="G168" s="2">
-        <v>40</v>
+        <v>127</v>
       </c>
       <c r="H168" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A169" s="2" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B169" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="C169" s="2" t="s">
         <v>323</v>
@@ -6174,24 +6177,24 @@
         <v>1</v>
       </c>
       <c r="E169" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F169" s="2">
-        <v>5320332</v>
+        <v>1830239</v>
       </c>
       <c r="G169" s="2">
-        <v>127</v>
+        <v>18</v>
       </c>
       <c r="H169" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A170" s="2" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="B170" s="2" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C170" s="2" t="s">
         <v>323</v>
@@ -6200,27 +6203,27 @@
         <v>1</v>
       </c>
       <c r="E170" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F170" s="2">
-        <v>1830239</v>
+        <v>5320332</v>
       </c>
       <c r="G170" s="2">
-        <v>18</v>
+        <v>181</v>
       </c>
       <c r="H170" s="2">
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A171" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B171" s="2" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C171" s="2" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="D171" s="2">
         <v>1</v>
@@ -6232,7 +6235,7 @@
         <v>5320332</v>
       </c>
       <c r="G171" s="2">
-        <v>181</v>
+        <v>95</v>
       </c>
       <c r="H171" s="2">
         <v>0</v>
@@ -6240,13 +6243,13 @@
     </row>
     <row r="172" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A172" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B172" s="2" t="s">
         <v>325</v>
       </c>
       <c r="C172" s="2" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D172" s="2">
         <v>1</v>
@@ -6258,7 +6261,7 @@
         <v>5320332</v>
       </c>
       <c r="G172" s="2">
-        <v>95</v>
+        <v>146</v>
       </c>
       <c r="H172" s="2">
         <v>0</v>
@@ -6269,22 +6272,22 @@
         <v>21</v>
       </c>
       <c r="B173" s="2" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C173" s="2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D173" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E173" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F173" s="2">
-        <v>5320332</v>
+        <v>1112262</v>
       </c>
       <c r="G173" s="2">
-        <v>146</v>
+        <v>55</v>
       </c>
       <c r="H173" s="2">
         <v>0</v>
@@ -6295,22 +6298,22 @@
         <v>21</v>
       </c>
       <c r="B174" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C174" s="2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="D174" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E174" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F174" s="2">
-        <v>1112262</v>
+        <v>1029126</v>
       </c>
       <c r="G174" s="2">
-        <v>55</v>
+        <v>128</v>
       </c>
       <c r="H174" s="2">
         <v>0</v>
@@ -6321,10 +6324,10 @@
         <v>21</v>
       </c>
       <c r="B175" s="2" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C175" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="D175" s="2">
         <v>3</v>
@@ -6336,7 +6339,7 @@
         <v>1029126</v>
       </c>
       <c r="G175" s="2">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="H175" s="2">
         <v>0</v>
@@ -6347,22 +6350,22 @@
         <v>21</v>
       </c>
       <c r="B176" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="C176" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="D176" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E176" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F176" s="2">
-        <v>1029126</v>
+        <v>1932179</v>
       </c>
       <c r="G176" s="2">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="H176" s="2">
         <v>0</v>
@@ -6370,13 +6373,13 @@
     </row>
     <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A177" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B177" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C177" s="2" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D177" s="2">
         <v>4</v>
@@ -6385,10 +6388,10 @@
         <v>13</v>
       </c>
       <c r="F177" s="2">
-        <v>1932179</v>
+        <v>2903204</v>
       </c>
       <c r="G177" s="2">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="H177" s="2">
         <v>0</v>
@@ -6396,25 +6399,25 @@
     </row>
     <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A178" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="B178" s="2" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C178" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="D178" s="2">
         <v>4</v>
       </c>
       <c r="E178" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F178" s="2">
-        <v>2903204</v>
+        <v>1086552</v>
       </c>
       <c r="G178" s="2">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="H178" s="2">
         <v>0</v>
@@ -6422,25 +6425,25 @@
     </row>
     <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A179" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B179" s="2" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="C179" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="D179" s="2">
         <v>4</v>
       </c>
       <c r="E179" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F179" s="2">
-        <v>1086552</v>
+        <v>4321939</v>
       </c>
       <c r="G179" s="2">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="H179" s="2">
         <v>0</v>
@@ -6448,25 +6451,25 @@
     </row>
     <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A180" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B180" s="2" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C180" s="2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="D180" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E180" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F180" s="2">
-        <v>4321939</v>
+        <v>2137934</v>
       </c>
       <c r="G180" s="2">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="H180" s="2">
         <v>0</v>
@@ -6474,25 +6477,25 @@
     </row>
     <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A181" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B181" s="2" t="s">
-        <v>342</v>
+        <v>192</v>
       </c>
       <c r="C181" s="2" t="s">
-        <v>343</v>
+        <v>193</v>
       </c>
       <c r="D181" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E181" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F181" s="2">
-        <v>2137934</v>
+        <v>2576518</v>
       </c>
       <c r="G181" s="2">
-        <v>84</v>
+        <v>15</v>
       </c>
       <c r="H181" s="2">
         <v>0</v>
@@ -6500,25 +6503,25 @@
     </row>
     <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A182" s="2" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B182" s="2" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="C182" s="2" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D182" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E182" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F182" s="2">
-        <v>3371830</v>
+        <v>2446060</v>
       </c>
       <c r="G182" s="2">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H182" s="2">
         <v>0</v>
@@ -6526,25 +6529,25 @@
     </row>
     <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A183" s="2" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="B183" s="2" t="s">
-        <v>346</v>
+        <v>224</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>347</v>
+        <v>225</v>
       </c>
       <c r="D183" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E183" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F183" s="2">
-        <v>2446060</v>
+        <v>5299061</v>
       </c>
       <c r="G183" s="2">
-        <v>6</v>
+        <v>19</v>
       </c>
       <c r="H183" s="2">
         <v>0</v>
@@ -6552,16 +6555,16 @@
     </row>
     <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A184" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B184" s="2" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D184" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E184" s="2" t="s">
         <v>13</v>
@@ -6570,15 +6573,15 @@
         <v>2832797</v>
       </c>
       <c r="G184" s="2">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="H184" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A185" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B185" s="2" t="s">
         <v>350</v>
@@ -6596,7 +6599,7 @@
         <v>2832797</v>
       </c>
       <c r="G185" s="2">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H185" s="2">
         <v>0</v>
@@ -6604,25 +6607,25 @@
     </row>
     <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A186" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B186" s="2" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="C186" s="2" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="D186" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E186" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F186" s="2">
-        <v>2832797</v>
+        <v>4721220</v>
       </c>
       <c r="G186" s="2">
-        <v>6</v>
+        <v>73</v>
       </c>
       <c r="H186" s="2">
         <v>0</v>
@@ -6630,39 +6633,39 @@
     </row>
     <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A187" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B187" s="2" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C187" s="2" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="D187" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E187" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F187" s="2">
-        <v>4721220</v>
+        <v>7248701</v>
       </c>
       <c r="G187" s="2">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="H187" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A188" s="2" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="B188" s="2" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C188" s="2" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D188" s="2">
         <v>4</v>
@@ -6671,62 +6674,62 @@
         <v>13</v>
       </c>
       <c r="F188" s="2">
-        <v>7248701</v>
+        <v>2923606</v>
       </c>
       <c r="G188" s="2">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="H188" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A189" s="2" t="s">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="B189" s="2" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C189" s="2" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="D189" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E189" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F189" s="2">
-        <v>2923606</v>
+        <v>3143825</v>
       </c>
       <c r="G189" s="2">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="H189" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A190" s="2" t="s">
-        <v>7</v>
+        <v>24</v>
       </c>
       <c r="B190" s="2" t="s">
-        <v>358</v>
+        <v>348</v>
       </c>
       <c r="C190" s="2" t="s">
-        <v>359</v>
+        <v>349</v>
       </c>
       <c r="D190" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E190" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F190" s="2">
-        <v>3143825</v>
+        <v>2832797</v>
       </c>
       <c r="G190" s="2">
-        <v>84</v>
+        <v>20</v>
       </c>
       <c r="H190" s="2">
         <v>1</v>
@@ -6734,7 +6737,7 @@
     </row>
     <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A191" s="2" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="B191" s="2" t="s">
         <v>360</v>
@@ -6743,16 +6746,16 @@
         <v>361</v>
       </c>
       <c r="D191" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E191" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F191" s="2">
-        <v>5318224</v>
+        <v>3435711</v>
       </c>
       <c r="G191" s="2">
-        <v>54</v>
+        <v>42</v>
       </c>
       <c r="H191" s="2">
         <v>0</v>
@@ -6769,24 +6772,24 @@
         <v>363</v>
       </c>
       <c r="D192" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E192" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F192" s="2">
-        <v>3435711</v>
+        <v>1267061</v>
       </c>
       <c r="G192" s="2">
-        <v>42</v>
+        <v>102</v>
       </c>
       <c r="H192" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A193" s="2" t="s">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="B193" s="2" t="s">
         <v>364</v>
@@ -6795,24 +6798,24 @@
         <v>365</v>
       </c>
       <c r="D193" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E193" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F193" s="2">
-        <v>1267061</v>
+        <v>2757489</v>
       </c>
       <c r="G193" s="2">
-        <v>102</v>
+        <v>43</v>
       </c>
       <c r="H193" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A194" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B194" s="2" t="s">
         <v>366</v>
@@ -6827,10 +6830,10 @@
         <v>13</v>
       </c>
       <c r="F194" s="2">
-        <v>2757489</v>
+        <v>2092090</v>
       </c>
       <c r="G194" s="2">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="H194" s="2">
         <v>0</v>
@@ -6838,13 +6841,13 @@
     </row>
     <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A195" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B195" s="2" t="s">
-        <v>368</v>
+        <v>142</v>
       </c>
       <c r="C195" s="2" t="s">
-        <v>369</v>
+        <v>143</v>
       </c>
       <c r="D195" s="2">
         <v>4</v>
@@ -6853,10 +6856,10 @@
         <v>13</v>
       </c>
       <c r="F195" s="2">
-        <v>2092090</v>
+        <v>1502554</v>
       </c>
       <c r="G195" s="2">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="H195" s="2">
         <v>0</v>
@@ -6864,7 +6867,7 @@
     </row>
     <row r="196" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A196" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B196" s="2" t="s">
         <v>370</v>
@@ -6873,16 +6876,16 @@
         <v>371</v>
       </c>
       <c r="D196" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E196" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F196" s="2">
-        <v>1707115</v>
+        <v>1214802</v>
       </c>
       <c r="G196" s="2">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="H196" s="2">
         <v>0</v>
@@ -6890,25 +6893,25 @@
     </row>
     <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A197" s="2" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B197" s="2" t="s">
-        <v>372</v>
+        <v>416</v>
       </c>
       <c r="C197" s="2" t="s">
-        <v>373</v>
+        <v>417</v>
       </c>
       <c r="D197" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E197" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F197" s="2">
-        <v>1214802</v>
+        <v>3334973</v>
       </c>
       <c r="G197" s="2">
-        <v>97</v>
+        <v>18</v>
       </c>
       <c r="H197" s="2">
         <v>0</v>
@@ -6916,25 +6919,25 @@
     </row>
     <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A198" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B198" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C198" s="2" t="s">
         <v>374</v>
-      </c>
-      <c r="C198" s="2" t="s">
-        <v>373</v>
       </c>
       <c r="D198" s="2">
         <v>1</v>
       </c>
       <c r="E198" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F198" s="2">
-        <v>2554019</v>
+        <v>1098471</v>
       </c>
       <c r="G198" s="2">
-        <v>141</v>
+        <v>19</v>
       </c>
       <c r="H198" s="2">
         <v>0</v>
@@ -6942,7 +6945,7 @@
     </row>
     <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A199" s="2" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="B199" s="2" t="s">
         <v>375</v>
@@ -6951,16 +6954,16 @@
         <v>376</v>
       </c>
       <c r="D199" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E199" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F199" s="2">
-        <v>1098471</v>
+        <v>1410757</v>
       </c>
       <c r="G199" s="2">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="H199" s="2">
         <v>0</v>
@@ -6968,7 +6971,7 @@
     </row>
     <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A200" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B200" s="2" t="s">
         <v>377</v>
@@ -6977,16 +6980,16 @@
         <v>378</v>
       </c>
       <c r="D200" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E200" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F200" s="2">
-        <v>1410757</v>
+        <v>1198965</v>
       </c>
       <c r="G200" s="2">
-        <v>8</v>
+        <v>73</v>
       </c>
       <c r="H200" s="2">
         <v>0</v>
@@ -7009,10 +7012,10 @@
         <v>10</v>
       </c>
       <c r="F201" s="2">
-        <v>1198965</v>
+        <v>1561186</v>
       </c>
       <c r="G201" s="2">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="H201" s="2">
         <v>0</v>
@@ -7020,7 +7023,7 @@
     </row>
     <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A202" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B202" s="2" t="s">
         <v>381</v>
@@ -7032,13 +7035,13 @@
         <v>3</v>
       </c>
       <c r="E202" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F202" s="2">
-        <v>1561186</v>
+        <v>5475421</v>
       </c>
       <c r="G202" s="2">
-        <v>70</v>
+        <v>24</v>
       </c>
       <c r="H202" s="2">
         <v>0</v>
@@ -7046,25 +7049,25 @@
     </row>
     <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A203" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B203" s="2" t="s">
-        <v>383</v>
+        <v>344</v>
       </c>
       <c r="C203" s="2" t="s">
-        <v>384</v>
+        <v>345</v>
       </c>
       <c r="D203" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E203" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F203" s="2">
-        <v>5475421</v>
+        <v>3371830</v>
       </c>
       <c r="G203" s="2">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H203" s="2">
         <v>0</v>
@@ -7072,7 +7075,7 @@
     </row>
     <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A204" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B204" s="2" t="s">
         <v>385</v>
@@ -7081,16 +7084,16 @@
         <v>386</v>
       </c>
       <c r="D204" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E204" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F204" s="2">
-        <v>1235319</v>
+        <v>1587825</v>
       </c>
       <c r="G204" s="2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="H204" s="2">
         <v>0</v>
@@ -7098,22 +7101,22 @@
     </row>
     <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A205" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B205" s="2" t="s">
-        <v>387</v>
+        <v>25</v>
       </c>
       <c r="C205" s="2" t="s">
-        <v>388</v>
+        <v>26</v>
       </c>
       <c r="D205" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E205" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F205" s="2">
-        <v>1587825</v>
+        <v>1502554</v>
       </c>
       <c r="G205" s="2">
         <v>18</v>
@@ -7124,7 +7127,7 @@
     </row>
     <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A206" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B206" s="2" t="s">
         <v>389</v>
@@ -7133,24 +7136,24 @@
         <v>390</v>
       </c>
       <c r="D206" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E206" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F206" s="2">
-        <v>1235319</v>
+        <v>1047857</v>
       </c>
       <c r="G206" s="2">
-        <v>21</v>
+        <v>90</v>
       </c>
       <c r="H206" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A207" s="2" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="B207" s="2" t="s">
         <v>391</v>
@@ -7159,24 +7162,24 @@
         <v>392</v>
       </c>
       <c r="D207" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E207" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F207" s="2">
-        <v>1047857</v>
+        <v>1583231</v>
       </c>
       <c r="G207" s="2">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="H207" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="208" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A208" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="B208" s="2" t="s">
         <v>393</v>
@@ -7191,10 +7194,10 @@
         <v>10</v>
       </c>
       <c r="F208" s="2">
-        <v>1583231</v>
+        <v>2571190</v>
       </c>
       <c r="G208" s="2">
-        <v>73</v>
+        <v>96</v>
       </c>
       <c r="H208" s="2">
         <v>0</v>
@@ -7202,7 +7205,7 @@
     </row>
     <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A209" s="2" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="B209" s="2" t="s">
         <v>395</v>
@@ -7211,16 +7214,16 @@
         <v>396</v>
       </c>
       <c r="D209" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E209" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F209" s="2">
-        <v>2571190</v>
+        <v>4205238</v>
       </c>
       <c r="G209" s="2">
-        <v>96</v>
+        <v>18</v>
       </c>
       <c r="H209" s="2">
         <v>0</v>
@@ -7228,25 +7231,25 @@
     </row>
     <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A210" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B210" s="2" t="s">
         <v>397</v>
       </c>
       <c r="C210" s="2" t="s">
-        <v>398</v>
+        <v>396</v>
       </c>
       <c r="D210" s="2">
         <v>2</v>
       </c>
       <c r="E210" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F210" s="2">
-        <v>4205238</v>
+        <v>5856415</v>
       </c>
       <c r="G210" s="2">
-        <v>18</v>
+        <v>91</v>
       </c>
       <c r="H210" s="2">
         <v>0</v>
@@ -7254,25 +7257,25 @@
     </row>
     <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A211" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B211" s="2" t="s">
-        <v>399</v>
+        <v>274</v>
       </c>
       <c r="C211" s="2" t="s">
-        <v>398</v>
+        <v>276</v>
       </c>
       <c r="D211" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E211" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F211" s="2">
-        <v>5856415</v>
+        <v>1739868</v>
       </c>
       <c r="G211" s="2">
-        <v>91</v>
+        <v>159</v>
       </c>
       <c r="H211" s="2">
         <v>0</v>
@@ -7280,7 +7283,7 @@
     </row>
     <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A212" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B212" s="2" t="s">
         <v>400</v>
@@ -7295,10 +7298,10 @@
         <v>10</v>
       </c>
       <c r="F212" s="2">
-        <v>2994200</v>
+        <v>2458943</v>
       </c>
       <c r="G212" s="2">
-        <v>131</v>
+        <v>105</v>
       </c>
       <c r="H212" s="2">
         <v>0</v>
@@ -7315,16 +7318,16 @@
         <v>403</v>
       </c>
       <c r="D213" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E213" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F213" s="2">
-        <v>2458943</v>
+        <v>2234229</v>
       </c>
       <c r="G213" s="2">
-        <v>105</v>
+        <v>22</v>
       </c>
       <c r="H213" s="2">
         <v>0</v>
@@ -7332,7 +7335,7 @@
     </row>
     <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A214" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B214" s="2" t="s">
         <v>404</v>
@@ -7347,10 +7350,10 @@
         <v>13</v>
       </c>
       <c r="F214" s="2">
-        <v>2234229</v>
+        <v>1410757</v>
       </c>
       <c r="G214" s="2">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="H214" s="2">
         <v>0</v>
@@ -7358,7 +7361,7 @@
     </row>
     <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A215" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B215" s="2" t="s">
         <v>406</v>
@@ -7367,16 +7370,16 @@
         <v>407</v>
       </c>
       <c r="D215" s="2">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E215" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F215" s="2">
-        <v>1410757</v>
+        <v>5930518</v>
       </c>
       <c r="G215" s="2">
-        <v>8</v>
+        <v>36</v>
       </c>
       <c r="H215" s="2">
         <v>0</v>
@@ -7384,7 +7387,7 @@
     </row>
     <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A216" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B216" s="2" t="s">
         <v>408</v>
@@ -7393,16 +7396,16 @@
         <v>409</v>
       </c>
       <c r="D216" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E216" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F216" s="2">
-        <v>5930518</v>
+        <v>7208507</v>
       </c>
       <c r="G216" s="2">
-        <v>36</v>
+        <v>62</v>
       </c>
       <c r="H216" s="2">
         <v>0</v>
@@ -7410,7 +7413,7 @@
     </row>
     <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A217" s="2" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B217" s="2" t="s">
         <v>410</v>
@@ -7425,10 +7428,10 @@
         <v>13</v>
       </c>
       <c r="F217" s="2">
-        <v>7208507</v>
+        <v>1214802</v>
       </c>
       <c r="G217" s="2">
-        <v>62</v>
+        <v>31</v>
       </c>
       <c r="H217" s="2">
         <v>0</v>
@@ -7436,7 +7439,7 @@
     </row>
     <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A218" s="2" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="B218" s="2" t="s">
         <v>412</v>
@@ -7445,16 +7448,16 @@
         <v>413</v>
       </c>
       <c r="D218" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E218" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F218" s="2">
-        <v>1214802</v>
+        <v>2002083</v>
       </c>
       <c r="G218" s="2">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="H218" s="2">
         <v>0</v>
@@ -7462,7 +7465,7 @@
     </row>
     <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A219" s="2" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="B219" s="2" t="s">
         <v>414</v>
@@ -7477,10 +7480,10 @@
         <v>13</v>
       </c>
       <c r="F219" s="2">
-        <v>2002083</v>
+        <v>5856415</v>
       </c>
       <c r="G219" s="2">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="H219" s="2">
         <v>0</v>
@@ -7488,22 +7491,22 @@
     </row>
     <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A220" s="2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B220" s="2" t="s">
-        <v>416</v>
+        <v>194</v>
       </c>
       <c r="C220" s="2" t="s">
-        <v>417</v>
+        <v>195</v>
       </c>
       <c r="D220" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E220" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F220" s="2">
-        <v>5856415</v>
+        <v>1210302</v>
       </c>
       <c r="G220" s="2">
         <v>34</v>
@@ -7514,7 +7517,7 @@
     </row>
     <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A221" s="2" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="B221" s="2" t="s">
         <v>418</v>
@@ -7523,16 +7526,16 @@
         <v>419</v>
       </c>
       <c r="D221" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E221" s="2" t="s">
         <v>13</v>
       </c>
       <c r="F221" s="2">
-        <v>3334973</v>
+        <v>5213213</v>
       </c>
       <c r="G221" s="2">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="H221" s="2">
         <v>0</v>
@@ -7549,16 +7552,16 @@
         <v>421</v>
       </c>
       <c r="D222" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E222" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F222" s="2">
-        <v>5213213</v>
+        <v>1021641</v>
       </c>
       <c r="G222" s="2">
-        <v>24</v>
+        <v>130</v>
       </c>
       <c r="H222" s="2">
         <v>0</v>
@@ -7581,10 +7584,10 @@
         <v>10</v>
       </c>
       <c r="F223" s="2">
-        <v>1021641</v>
+        <v>2092090</v>
       </c>
       <c r="G223" s="2">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H223" s="2">
         <v>0</v>
@@ -7592,7 +7595,7 @@
     </row>
     <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A224" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B224" s="2" t="s">
         <v>424</v>
@@ -7601,16 +7604,16 @@
         <v>425</v>
       </c>
       <c r="D224" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E224" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F224" s="2">
-        <v>2092090</v>
+        <v>5997408</v>
       </c>
       <c r="G224" s="2">
-        <v>127</v>
+        <v>9</v>
       </c>
       <c r="H224" s="2">
         <v>0</v>
@@ -7618,7 +7621,7 @@
     </row>
     <row r="225" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A225" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B225" s="2" t="s">
         <v>426</v>
@@ -7630,13 +7633,13 @@
         <v>4</v>
       </c>
       <c r="E225" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F225" s="2">
-        <v>5997408</v>
+        <v>3524624</v>
       </c>
       <c r="G225" s="2">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="H225" s="2">
         <v>0</v>
@@ -7644,7 +7647,7 @@
     </row>
     <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A226" s="2" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B226" s="2" t="s">
         <v>428</v>
@@ -7653,16 +7656,16 @@
         <v>429</v>
       </c>
       <c r="D226" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E226" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="F226" s="2">
-        <v>3524624</v>
+        <v>1892200</v>
       </c>
       <c r="G226" s="2">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="H226" s="2">
         <v>0</v>
@@ -7670,7 +7673,7 @@
     </row>
     <row r="227" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
       <c r="A227" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B227" s="2" t="s">
         <v>430</v>
@@ -7682,41 +7685,15 @@
         <v>3</v>
       </c>
       <c r="E227" s="2" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F227" s="2">
-        <v>1892200</v>
+        <v>2977082</v>
       </c>
       <c r="G227" s="2">
-        <v>5</v>
+        <v>52</v>
       </c>
       <c r="H227" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="228" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
-      <c r="A228" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B228" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="C228" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="D228" s="2">
-        <v>3</v>
-      </c>
-      <c r="E228" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F228" s="2">
-        <v>2977082</v>
-      </c>
-      <c r="G228" s="2">
-        <v>52</v>
-      </c>
-      <c r="H228" s="2">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
room-time and room-utilization analysis done. TODO: daily deparment-year distribution analysis
</commit_message>
<xml_diff>
--- a/data/BerkData2.xlsx
+++ b/data/BerkData2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9e402f802124af4b/Masaüstü/Projects/Campus-Scheduling/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ercx2\Desktop\Scheduling Theory_02\Paper\scheduling\Campus-Scheduling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{2C943E96-C6E4-40C4-888D-FAADD3A22539}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73EF178F-B942-4E9E-B37E-B80A3349A76A}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63289AB0-56F6-47B5-BD19-022E00C6CFBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-17640" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1820" yWindow="1820" windowWidth="24460" windowHeight="12780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1467,21 +1467,9 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}" name="Table1" displayName="Table1" ref="A1:H227" totalsRowShown="0" headerRowDxfId="11" dataDxfId="9" headerRowBorderDxfId="10" tableBorderDxfId="8">
-  <autoFilter ref="A1:H227" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="EEM 370"/>
-        <filter val="FİZ 174"/>
-        <filter val="GIDA 324"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:H227" xr:uid="{4D257DAD-E412-40CE-835B-244614789DDA}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A8:H220">
     <sortCondition ref="B1:B227"/>
   </sortState>
@@ -1785,17 +1773,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H227"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.19921875" customWidth="1"/>
-    <col min="2" max="2" width="16.265625" customWidth="1"/>
-    <col min="3" max="3" width="37.46484375" customWidth="1"/>
-    <col min="5" max="5" width="10.265625" customWidth="1"/>
-    <col min="6" max="6" width="16.59765625" customWidth="1"/>
-    <col min="7" max="7" width="14.19921875" customWidth="1"/>
+    <col min="1" max="1" width="22.1796875" customWidth="1"/>
+    <col min="2" max="2" width="16.26953125" customWidth="1"/>
+    <col min="3" max="3" width="37.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="16.6328125" customWidth="1"/>
+    <col min="7" max="7" width="14.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1821,7 +1809,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
@@ -1847,7 +1835,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -1873,7 +1861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
@@ -1899,7 +1887,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>17</v>
       </c>
@@ -1925,7 +1913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>19</v>
       </c>
@@ -1951,7 +1939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>21</v>
       </c>
@@ -1977,7 +1965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>24</v>
       </c>
@@ -2003,7 +1991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
@@ -2029,7 +2017,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>21</v>
       </c>
@@ -2055,7 +2043,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>27</v>
       </c>
@@ -2081,7 +2069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -2107,7 +2095,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>27</v>
       </c>
@@ -2133,7 +2121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>21</v>
       </c>
@@ -2159,7 +2147,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>21</v>
       </c>
@@ -2185,7 +2173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>21</v>
       </c>
@@ -2211,7 +2199,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -2237,7 +2225,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>27</v>
       </c>
@@ -2263,7 +2251,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>24</v>
       </c>
@@ -2289,7 +2277,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>21</v>
       </c>
@@ -2315,7 +2303,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>24</v>
       </c>
@@ -2341,7 +2329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>24</v>
       </c>
@@ -2367,7 +2355,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
@@ -2393,7 +2381,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>14</v>
       </c>
@@ -2419,7 +2407,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>24</v>
       </c>
@@ -2445,7 +2433,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>17</v>
       </c>
@@ -2471,7 +2459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>19</v>
       </c>
@@ -2497,7 +2485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>21</v>
       </c>
@@ -2523,7 +2511,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>17</v>
       </c>
@@ -2549,7 +2537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>27</v>
       </c>
@@ -2575,7 +2563,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>19</v>
       </c>
@@ -2601,7 +2589,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>27</v>
       </c>
@@ -2627,7 +2615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>21</v>
       </c>
@@ -2653,7 +2641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>19</v>
       </c>
@@ -2679,7 +2667,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>21</v>
       </c>
@@ -2705,7 +2693,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>17</v>
       </c>
@@ -2731,7 +2719,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>7</v>
       </c>
@@ -2757,7 +2745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>7</v>
       </c>
@@ -2783,7 +2771,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>27</v>
       </c>
@@ -2809,7 +2797,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>7</v>
       </c>
@@ -2835,7 +2823,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>7</v>
       </c>
@@ -2861,7 +2849,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>7</v>
       </c>
@@ -2887,7 +2875,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>21</v>
       </c>
@@ -2913,7 +2901,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>14</v>
       </c>
@@ -2939,7 +2927,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>27</v>
       </c>
@@ -2965,7 +2953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>27</v>
       </c>
@@ -2991,7 +2979,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>7</v>
       </c>
@@ -3017,7 +3005,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>24</v>
       </c>
@@ -3043,7 +3031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>27</v>
       </c>
@@ -3069,7 +3057,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>7</v>
       </c>
@@ -3095,7 +3083,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>21</v>
       </c>
@@ -3121,7 +3109,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>21</v>
       </c>
@@ -3147,7 +3135,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>24</v>
       </c>
@@ -3173,7 +3161,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>7</v>
       </c>
@@ -3199,7 +3187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>24</v>
       </c>
@@ -3225,7 +3213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>14</v>
       </c>
@@ -3251,7 +3239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>19</v>
       </c>
@@ -3277,7 +3265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>21</v>
       </c>
@@ -3303,7 +3291,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>21</v>
       </c>
@@ -3329,7 +3317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>21</v>
       </c>
@@ -3355,7 +3343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>21</v>
       </c>
@@ -3381,7 +3369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>21</v>
       </c>
@@ -3407,7 +3395,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>24</v>
       </c>
@@ -3433,7 +3421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>21</v>
       </c>
@@ -3459,7 +3447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>27</v>
       </c>
@@ -3485,7 +3473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>14</v>
       </c>
@@ -3511,7 +3499,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>19</v>
       </c>
@@ -3537,7 +3525,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>24</v>
       </c>
@@ -3563,7 +3551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>21</v>
       </c>
@@ -3589,7 +3577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>21</v>
       </c>
@@ -3615,7 +3603,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>7</v>
       </c>
@@ -3641,7 +3629,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>24</v>
       </c>
@@ -3667,7 +3655,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>27</v>
       </c>
@@ -3693,7 +3681,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>19</v>
       </c>
@@ -3719,7 +3707,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>24</v>
       </c>
@@ -3745,7 +3733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>14</v>
       </c>
@@ -3771,7 +3759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>17</v>
       </c>
@@ -3797,7 +3785,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>24</v>
       </c>
@@ -3823,7 +3811,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>19</v>
       </c>
@@ -3849,7 +3837,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>21</v>
       </c>
@@ -3875,7 +3863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>27</v>
       </c>
@@ -3901,7 +3889,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>17</v>
       </c>
@@ -3927,7 +3915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>19</v>
       </c>
@@ -3953,7 +3941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>19</v>
       </c>
@@ -3979,7 +3967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>19</v>
       </c>
@@ -4005,7 +3993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>19</v>
       </c>
@@ -4031,7 +4019,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>19</v>
       </c>
@@ -4057,7 +4045,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>19</v>
       </c>
@@ -4083,7 +4071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>19</v>
       </c>
@@ -4109,7 +4097,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>19</v>
       </c>
@@ -4135,7 +4123,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>19</v>
       </c>
@@ -4161,7 +4149,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>19</v>
       </c>
@@ -4187,7 +4175,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>14</v>
       </c>
@@ -4213,7 +4201,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>21</v>
       </c>
@@ -4239,7 +4227,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>24</v>
       </c>
@@ -4265,7 +4253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>24</v>
       </c>
@@ -4291,7 +4279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>17</v>
       </c>
@@ -4317,7 +4305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>27</v>
       </c>
@@ -4343,7 +4331,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>24</v>
       </c>
@@ -4369,7 +4357,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>14</v>
       </c>
@@ -4395,7 +4383,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>27</v>
       </c>
@@ -4421,7 +4409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>7</v>
       </c>
@@ -4447,7 +4435,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>7</v>
       </c>
@@ -4473,7 +4461,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>7</v>
       </c>
@@ -4499,7 +4487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>7</v>
       </c>
@@ -4525,7 +4513,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>7</v>
       </c>
@@ -4551,7 +4539,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>7</v>
       </c>
@@ -4577,7 +4565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>21</v>
       </c>
@@ -4603,7 +4591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>21</v>
       </c>
@@ -4629,7 +4617,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>21</v>
       </c>
@@ -4655,7 +4643,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>24</v>
       </c>
@@ -4681,7 +4669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>7</v>
       </c>
@@ -4707,7 +4695,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
         <v>24</v>
       </c>
@@ -4733,7 +4721,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>14</v>
       </c>
@@ -4759,7 +4747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
         <v>19</v>
       </c>
@@ -4785,7 +4773,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
         <v>14</v>
       </c>
@@ -4811,7 +4799,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>27</v>
       </c>
@@ -4837,7 +4825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>24</v>
       </c>
@@ -4863,7 +4851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>24</v>
       </c>
@@ -4889,7 +4877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>17</v>
       </c>
@@ -4915,7 +4903,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A121" s="2" t="s">
         <v>17</v>
       </c>
@@ -4941,7 +4929,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="122" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
         <v>17</v>
       </c>
@@ -4967,7 +4955,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
         <v>19</v>
       </c>
@@ -4993,7 +4981,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
         <v>7</v>
       </c>
@@ -5019,7 +5007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A125" s="2" t="s">
         <v>14</v>
       </c>
@@ -5045,7 +5033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>27</v>
       </c>
@@ -5071,7 +5059,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="127" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
         <v>19</v>
       </c>
@@ -5097,7 +5085,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="128" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
         <v>24</v>
       </c>
@@ -5123,7 +5111,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="129" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A129" s="2" t="s">
         <v>17</v>
       </c>
@@ -5149,7 +5137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="130" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
         <v>14</v>
       </c>
@@ -5175,7 +5163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="131" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
         <v>7</v>
       </c>
@@ -5201,7 +5189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="132" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="132" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
         <v>21</v>
       </c>
@@ -5227,7 +5215,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="133" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="133" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
         <v>14</v>
       </c>
@@ -5253,7 +5241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
         <v>24</v>
       </c>
@@ -5279,7 +5267,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A135" s="2" t="s">
         <v>17</v>
       </c>
@@ -5305,7 +5293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
         <v>17</v>
       </c>
@@ -5331,7 +5319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
         <v>24</v>
       </c>
@@ -5357,7 +5345,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>24</v>
       </c>
@@ -5383,7 +5371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A139" s="2" t="s">
         <v>14</v>
       </c>
@@ -5409,7 +5397,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
         <v>17</v>
       </c>
@@ -5435,7 +5423,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A141" s="2" t="s">
         <v>24</v>
       </c>
@@ -5461,7 +5449,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A142" s="2" t="s">
         <v>19</v>
       </c>
@@ -5487,7 +5475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="143" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A143" s="2" t="s">
         <v>7</v>
       </c>
@@ -5513,7 +5501,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="144" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
         <v>27</v>
       </c>
@@ -5539,7 +5527,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A145" s="2" t="s">
         <v>21</v>
       </c>
@@ -5565,7 +5553,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
         <v>24</v>
       </c>
@@ -5591,7 +5579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="147" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="147" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A147" s="2" t="s">
         <v>17</v>
       </c>
@@ -5617,7 +5605,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="148" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A148" s="2" t="s">
         <v>7</v>
       </c>
@@ -5643,7 +5631,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A149" s="2" t="s">
         <v>21</v>
       </c>
@@ -5669,7 +5657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="150" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
         <v>21</v>
       </c>
@@ -5695,7 +5683,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="151" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="151" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
         <v>14</v>
       </c>
@@ -5721,7 +5709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="152" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="152" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A152" s="2" t="s">
         <v>17</v>
       </c>
@@ -5747,7 +5735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="153" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
         <v>7</v>
       </c>
@@ -5773,7 +5761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="154" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A154" s="2" t="s">
         <v>19</v>
       </c>
@@ -5799,7 +5787,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="155" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A155" s="2" t="s">
         <v>14</v>
       </c>
@@ -5825,7 +5813,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="156" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="156" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
         <v>24</v>
       </c>
@@ -5851,7 +5839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
         <v>24</v>
       </c>
@@ -5877,7 +5865,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
         <v>24</v>
       </c>
@@ -5903,7 +5891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A159" s="2" t="s">
         <v>14</v>
       </c>
@@ -5929,7 +5917,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A160" s="2" t="s">
         <v>14</v>
       </c>
@@ -5955,7 +5943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
         <v>27</v>
       </c>
@@ -5981,7 +5969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="162" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
         <v>17</v>
       </c>
@@ -6007,7 +5995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
         <v>19</v>
       </c>
@@ -6033,7 +6021,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
         <v>21</v>
       </c>
@@ -6059,7 +6047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
         <v>19</v>
       </c>
@@ -6085,7 +6073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A166" s="2" t="s">
         <v>7</v>
       </c>
@@ -6111,7 +6099,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A167" s="2" t="s">
         <v>19</v>
       </c>
@@ -6137,7 +6125,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A168" s="2" t="s">
         <v>7</v>
       </c>
@@ -6163,7 +6151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A169" s="2" t="s">
         <v>27</v>
       </c>
@@ -6189,7 +6177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="170" spans="1:8" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A170" s="2" t="s">
         <v>21</v>
       </c>
@@ -6215,7 +6203,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
         <v>7</v>
       </c>
@@ -6241,7 +6229,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="172" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
         <v>21</v>
       </c>
@@ -6267,7 +6255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
         <v>21</v>
       </c>
@@ -6293,7 +6281,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
         <v>21</v>
       </c>
@@ -6319,7 +6307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A175" s="2" t="s">
         <v>21</v>
       </c>
@@ -6345,7 +6333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
         <v>21</v>
       </c>
@@ -6371,7 +6359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
         <v>7</v>
       </c>
@@ -6397,7 +6385,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
         <v>19</v>
       </c>
@@ -6423,7 +6411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A179" s="2" t="s">
         <v>21</v>
       </c>
@@ -6449,7 +6437,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
         <v>19</v>
       </c>
@@ -6475,7 +6463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
         <v>24</v>
       </c>
@@ -6501,7 +6489,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
         <v>17</v>
       </c>
@@ -6527,7 +6515,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
         <v>24</v>
       </c>
@@ -6553,7 +6541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A184" s="2" t="s">
         <v>27</v>
       </c>
@@ -6579,7 +6567,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A185" s="2" t="s">
         <v>17</v>
       </c>
@@ -6605,7 +6593,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="186" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A186" s="2" t="s">
         <v>21</v>
       </c>
@@ -6631,7 +6619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="187" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
         <v>7</v>
       </c>
@@ -6657,7 +6645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="188" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
         <v>21</v>
       </c>
@@ -6683,7 +6671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="189" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="189" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
         <v>7</v>
       </c>
@@ -6709,7 +6697,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="190" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
         <v>24</v>
       </c>
@@ -6735,7 +6723,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
         <v>7</v>
       </c>
@@ -6761,7 +6749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
         <v>7</v>
       </c>
@@ -6787,7 +6775,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A193" s="2" t="s">
         <v>19</v>
       </c>
@@ -6813,7 +6801,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A194" s="2" t="s">
         <v>14</v>
       </c>
@@ -6839,7 +6827,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="195" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A195" s="2" t="s">
         <v>24</v>
       </c>
@@ -6865,7 +6853,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="196" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
         <v>14</v>
       </c>
@@ -6891,7 +6879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
         <v>24</v>
       </c>
@@ -6917,7 +6905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
         <v>27</v>
       </c>
@@ -6943,7 +6931,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="199" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A199" s="2" t="s">
         <v>17</v>
       </c>
@@ -6969,7 +6957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
         <v>14</v>
       </c>
@@ -6995,7 +6983,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
         <v>14</v>
       </c>
@@ -7021,7 +7009,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="202" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A202" s="2" t="s">
         <v>19</v>
       </c>
@@ -7047,7 +7035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="203" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
         <v>24</v>
       </c>
@@ -7073,7 +7061,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A204" s="2" t="s">
         <v>27</v>
       </c>
@@ -7099,7 +7087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A205" s="2" t="s">
         <v>24</v>
       </c>
@@ -7125,7 +7113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="206" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A206" s="2" t="s">
         <v>19</v>
       </c>
@@ -7151,7 +7139,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="207" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
         <v>14</v>
       </c>
@@ -7177,7 +7165,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="208" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="208" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A208" s="2" t="s">
         <v>19</v>
       </c>
@@ -7203,7 +7191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="209" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
         <v>27</v>
       </c>
@@ -7229,7 +7217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
         <v>19</v>
       </c>
@@ -7255,7 +7243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A211" s="2" t="s">
         <v>24</v>
       </c>
@@ -7281,7 +7269,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A212" s="2" t="s">
         <v>14</v>
       </c>
@@ -7307,7 +7295,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A213" s="2" t="s">
         <v>14</v>
       </c>
@@ -7333,7 +7321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A214" s="2" t="s">
         <v>17</v>
       </c>
@@ -7359,7 +7347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A215" s="2" t="s">
         <v>19</v>
       </c>
@@ -7385,7 +7373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A216" s="2" t="s">
         <v>21</v>
       </c>
@@ -7411,7 +7399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A217" s="2" t="s">
         <v>14</v>
       </c>
@@ -7437,7 +7425,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="218" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
         <v>27</v>
       </c>
@@ -7463,7 +7451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A219" s="2" t="s">
         <v>19</v>
       </c>
@@ -7489,7 +7477,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A220" s="2" t="s">
         <v>24</v>
       </c>
@@ -7515,7 +7503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A221" s="2" t="s">
         <v>14</v>
       </c>
@@ -7541,7 +7529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A222" s="2" t="s">
         <v>14</v>
       </c>
@@ -7567,7 +7555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
         <v>14</v>
       </c>
@@ -7593,7 +7581,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="224" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A224" s="2" t="s">
         <v>17</v>
       </c>
@@ -7619,7 +7607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="225" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="225" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A225" s="2" t="s">
         <v>14</v>
       </c>
@@ -7645,7 +7633,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A226" s="2" t="s">
         <v>17</v>
       </c>
@@ -7671,7 +7659,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="227" spans="1:8" hidden="1" x14ac:dyDescent="0.45">
+    <row r="227" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A227" s="2" t="s">
         <v>14</v>
       </c>

</xml_diff>